<commit_message>
I was able to read the data from the excel file using pandas (and openxl) to answer some of the form questions. That's good. Streamlining the control flow so that it does everything automatically until it is unable to fill out a form element. i.e. anything other than a label fails. Detect that, stop automation.
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
   <si>
     <t>Question</t>
   </si>
@@ -67,6 +67,27 @@
   </si>
   <si>
     <t>no, I have a DHS Public Trust</t>
+  </si>
+  <si>
+    <t>select-one</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t>Weekday</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Anytime (8am - 9pm)</t>
+  </si>
+  <si>
+    <t>button</t>
+  </si>
+  <si>
+    <t>Continue</t>
   </si>
 </sst>
 </file>
@@ -397,7 +418,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -405,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.42578125" customWidth="1"/>
@@ -512,13 +533,49 @@
         <v>14</v>
       </c>
     </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576 B1 B1">
-      <formula1>"radio, select, text"</formula1>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B10 B12:B1048576">
+      <formula1>"radio, select, text, select-one, button"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="information" allowBlank="1" showInputMessage="1" sqref="C1:C1048576">
+    <dataValidation type="list" errorStyle="information" allowBlank="1" showInputMessage="1" sqref="C1:C1048576 A12">
       <formula1>"yes, no"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11">
+      <formula1>"radio, select, text, select-one"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
I need to find a more efficient way to directly read a label and thereby go directly to the associated input element instead of iterating through everything. Next step is to check for text type input elements
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="24">
   <si>
     <t>Question</t>
   </si>
@@ -88,6 +88,12 @@
   </si>
   <si>
     <t>Continue</t>
+  </si>
+  <si>
+    <t>able to relocate</t>
+  </si>
+  <si>
+    <t>Doesn't apply</t>
   </si>
 </sst>
 </file>
@@ -418,7 +424,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -426,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.42578125" customWidth="1"/>
@@ -566,17 +572,29 @@
         <v>21</v>
       </c>
     </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B10 B12:B1048576">
       <formula1>"radio, select, text, select-one, button"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="information" allowBlank="1" showInputMessage="1" sqref="C1:C1048576 A12">
+    <dataValidation type="list" errorStyle="information" allowBlank="1" showInputMessage="1" sqref="C1:C1048576">
       <formula1>"yes, no"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11">
       <formula1>"radio, select, text, select-one"</formula1>
     </dataValidation>
+    <dataValidation errorStyle="information" allowBlank="1" showInputMessage="1" sqref="A12"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
print out the last rows of QTV_excel file to show recent changes on update. Also looks like I need to stick with using the xpath to access an element directly for proper automation using Selenium. Next step: store or 'save' the current implementation in a function, develop a more direct/foolproof implementation using XPath and better analysis of DOM hierarchy. Think jQuery- you did this before!
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="35">
   <si>
     <t>Question</t>
   </si>
@@ -94,6 +94,39 @@
   </si>
   <si>
     <t>Doesn't apply</t>
+  </si>
+  <si>
+    <t>How many years of Robotic Process Automation</t>
+  </si>
+  <si>
+    <t>While I haven’t used UiPath directly, I have hands-on experience building automation workflows using Python and scripting tools to perform tasks similar to what UiPath enables. At MobileFrontiers, I wrote automation scripts for containerized environments using Docker, streamlining repetitive setup and deployment processes. In another project, I developed a Python-based GUI tool using Selenium, Tkinter, and pandas to automate web form submissions, data extraction, and Excel integration — all user-controlled through a front-end interface. These solutions handled decision logic, error handling, and multi-step workflows, closely aligning with the goals of RPA tools like UiPath. I’m confident I can apply these skills to UiPath or similar platforms with minimal ramp-up time.</t>
+  </si>
+  <si>
+    <t>Describe your experience with UiPath or similar technologies</t>
+  </si>
+  <si>
+    <t>position requires US citizenship</t>
+  </si>
+  <si>
+    <t>Yes- and I have a DHS Public Trust</t>
+  </si>
+  <si>
+    <t>How many years of Java experience do you have?</t>
+  </si>
+  <si>
+    <t>How many years of AWS experience do you have?</t>
+  </si>
+  <si>
+    <t>How many years of Microservices experience do you have?</t>
+  </si>
+  <si>
+    <t>How many years of MongoDB experience do you have?</t>
+  </si>
+  <si>
+    <t>required citizenship status is US Citizen</t>
+  </si>
+  <si>
+    <t>Apply anyway</t>
   </si>
 </sst>
 </file>
@@ -432,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.42578125" customWidth="1"/>
@@ -581,6 +614,105 @@
       </c>
       <c r="C13" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
To much nonsense with the random values they assign to the radio input elements. Instead, I should find the label, and then the input element nested inside with XPath. Please re-write whatever nonsense algorithm I wrote for iterating over the elements
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$29</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
   <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="50">
   <si>
     <t>Question</t>
   </si>
@@ -127,6 +127,51 @@
   </si>
   <si>
     <t>Apply anyway</t>
+  </si>
+  <si>
+    <t>When are you available to start</t>
+  </si>
+  <si>
+    <t>Anytime</t>
+  </si>
+  <si>
+    <t>How many years of HP Non Stop / Tandem experience do you have?</t>
+  </si>
+  <si>
+    <t>How many years of Python experience do you have?</t>
+  </si>
+  <si>
+    <t>How many years of airflow experience do you have?</t>
+  </si>
+  <si>
+    <t>How many years of applicable experience do you have?</t>
+  </si>
+  <si>
+    <t>What is your expected salary?</t>
+  </si>
+  <si>
+    <t>Do you have a TS/SCI with CI poly?</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Do you have an active Top Secret security clearance?</t>
+  </si>
+  <si>
+    <t>Are you eligible to work in the United States?</t>
+  </si>
+  <si>
+    <t>require any immigration related support or sponsorship</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> requires a minimum of three(3) years of physical presence in the U.S.</t>
+  </si>
+  <si>
+    <t>Are you able to perform the functions of the job, with or without reasonable accomodations?</t>
+  </si>
+  <si>
+    <t>Are you a protected Veteran?</t>
   </si>
 </sst>
 </file>
@@ -457,7 +502,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -465,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.42578125" customWidth="1"/>
@@ -596,84 +641,84 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" t="s">
-        <v>23</v>
+        <v>12</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
-      <c r="C14">
-        <v>2</v>
+      <c r="C14" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
         <v>12</v>
       </c>
-      <c r="C16" t="s">
-        <v>28</v>
+      <c r="C16">
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
         <v>12</v>
       </c>
       <c r="C17">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
         <v>12</v>
       </c>
       <c r="C18">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
@@ -684,49 +729,192 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B20" t="s">
         <v>12</v>
       </c>
-      <c r="C20">
-        <v>1</v>
+      <c r="C20" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B21" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
         <v>20</v>
       </c>
-      <c r="C22" t="s">
-        <v>34</v>
+      <c r="C23" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B10 B12:B1048576">
+    <dataValidation errorStyle="information" allowBlank="1" showInputMessage="1" sqref="A23"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B10 B12:B23 B25:B1048576">
       <formula1>"radio, select, text, select-one, button"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="information" allowBlank="1" showInputMessage="1" sqref="C1:C1048576">
+    <dataValidation type="list" errorStyle="information" allowBlank="1" showInputMessage="1" sqref="C1:C23 C25:C1048576">
       <formula1>"yes, no"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11">
       <formula1>"radio, select, text, select-one"</formula1>
     </dataValidation>
-    <dataValidation errorStyle="information" allowBlank="1" showInputMessage="1" sqref="A12"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
So it more or less works, I suppose the next step is to wrap each step as a function and add some try-catching so I can keep going even if webdriver gets a stale head. Then the next step probably is to make a class for the automation, which will function different according to the website webdriver is on. So like a 'profile' for each website
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="61">
   <si>
     <t>Question</t>
   </si>
@@ -172,6 +172,39 @@
   </si>
   <si>
     <t>Are you a protected Veteran?</t>
+  </si>
+  <si>
+    <t>Do you currently have a relative or spouse working at</t>
+  </si>
+  <si>
+    <t>Have you previously been employed by</t>
+  </si>
+  <si>
+    <t>Are you authorized to work in the US?</t>
+  </si>
+  <si>
+    <t>Do you need, or will you need in the future, any immigration-related support or sponsorship</t>
+  </si>
+  <si>
+    <t>Are you able to obtain a Government Clearance</t>
+  </si>
+  <si>
+    <t>What are your salary expectations?</t>
+  </si>
+  <si>
+    <t>Do you have an active government clearance? Please list specifics in the text field</t>
+  </si>
+  <si>
+    <t>Yes, DHS Public Trust</t>
+  </si>
+  <si>
+    <t>Do you have 8+ years of Microsoft Power Platform</t>
+  </si>
+  <si>
+    <t>Do you have 5+ years of Microsoft Power Platform</t>
+  </si>
+  <si>
+    <t>Do you have 1 or more of the following certifications?</t>
   </si>
 </sst>
 </file>
@@ -502,7 +535,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -510,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.42578125" customWidth="1"/>
@@ -900,6 +933,116 @@
         <v>9</v>
       </c>
       <c r="C35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>53</v>
+      </c>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>55</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>56</v>
+      </c>
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>58</v>
+      </c>
+      <c r="B43" t="s">
+        <v>9</v>
+      </c>
+      <c r="C43" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>59</v>
+      </c>
+      <c r="B44" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>60</v>
+      </c>
+      <c r="B45" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>

<commit_message>
I structure the code to be more object oriented. There are so many edge cases though. Randomly indeed decides to use a fieldset instead on certain pages. Anyways, I suppose next steps are: 1. handing of each target element type could be encapsulated as a function 2. Once the run() function in automate.py is more modularized by #1, I could tackle other types of webpages to automate.
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="83">
   <si>
     <t>Question</t>
   </si>
@@ -205,6 +205,72 @@
   </si>
   <si>
     <t>Do you have 1 or more of the following certifications?</t>
+  </si>
+  <si>
+    <t>Do you have a valid US Citizenship</t>
+  </si>
+  <si>
+    <t>How many years of Linux Administration experience do you have?</t>
+  </si>
+  <si>
+    <t>applied DevOps professional experience do you have?</t>
+  </si>
+  <si>
+    <t>Please list any relevant certifications you hold</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>Total years of relative experience?</t>
+  </si>
+  <si>
+    <t>2+</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>Bachelors Degree</t>
+  </si>
+  <si>
+    <t>active DoD clearance</t>
+  </si>
+  <si>
+    <t>Clearance Level</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Race</t>
+  </si>
+  <si>
+    <t>Asian</t>
+  </si>
+  <si>
+    <t>Veteran Status</t>
+  </si>
+  <si>
+    <t>I am not a veteran</t>
+  </si>
+  <si>
+    <t>Protected Veteran Status</t>
+  </si>
+  <si>
+    <t>I am not a protected veteran</t>
+  </si>
+  <si>
+    <t>Disability Status</t>
+  </si>
+  <si>
+    <t>No, I do not have a disability and have not had one in the past</t>
   </si>
 </sst>
 </file>
@@ -535,7 +601,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -543,7 +609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.42578125" customWidth="1"/>
@@ -1044,6 +1110,149 @@
       </c>
       <c r="C45" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>61</v>
+      </c>
+      <c r="B46" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>66</v>
+      </c>
+      <c r="B50" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
+        <v>68</v>
+      </c>
+      <c r="B51" t="s">
+        <v>9</v>
+      </c>
+      <c r="C51" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
+        <v>70</v>
+      </c>
+      <c r="B52" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>71</v>
+      </c>
+      <c r="B53" t="s">
+        <v>9</v>
+      </c>
+      <c r="C53" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>73</v>
+      </c>
+      <c r="B54" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>75</v>
+      </c>
+      <c r="B55" t="s">
+        <v>15</v>
+      </c>
+      <c r="C55" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
+        <v>77</v>
+      </c>
+      <c r="B56" t="s">
+        <v>9</v>
+      </c>
+      <c r="C56" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
+        <v>79</v>
+      </c>
+      <c r="B57" t="s">
+        <v>9</v>
+      </c>
+      <c r="C57" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>81</v>
+      </c>
+      <c r="B58" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
page_visible_info: Improved readability of page_visible_info terminal output for viewing page, also used match case for improved code readability (perhaps?), added 'legend' as one of the visible HTML tags to search for.
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="85">
   <si>
     <t>Question</t>
   </si>
@@ -271,6 +271,12 @@
   </si>
   <si>
     <t>No, I do not have a disability and have not had one in the past</t>
+  </si>
+  <si>
+    <t>Are you located in Arizona? *</t>
+  </si>
+  <si>
+    <t>How many years of modern JavaScript experience do you have?</t>
   </si>
 </sst>
 </file>
@@ -609,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.42578125" customWidth="1"/>
@@ -1253,6 +1259,28 @@
       </c>
       <c r="C58" t="s">
         <v>82</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>83</v>
+      </c>
+      <c r="B59" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>84</v>
+      </c>
+      <c r="B60" t="s">
+        <v>12</v>
+      </c>
+      <c r="C60">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Got the basic UI setup for adding an entry into excel throught the Window GUI
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="96">
   <si>
     <t>Question</t>
   </si>
@@ -33,12 +33,6 @@
     <t>Value</t>
   </si>
   <si>
-    <t>Are you a US Citizen</t>
-  </si>
-  <si>
-    <t>are you a u.s. citizen</t>
-  </si>
-  <si>
     <t>Do you have a Bachelor's Degree</t>
   </si>
   <si>
@@ -147,9 +141,6 @@
     <t>How many years of applicable experience do you have?</t>
   </si>
   <si>
-    <t>What is your expected salary?</t>
-  </si>
-  <si>
     <t>Do you have a TS/SCI with CI poly?</t>
   </si>
   <si>
@@ -277,6 +268,48 @@
   </si>
   <si>
     <t>How many years of modern JavaScript experience do you have?</t>
+  </si>
+  <si>
+    <t>US Citizen</t>
+  </si>
+  <si>
+    <t>u.s. citizen</t>
+  </si>
+  <si>
+    <t>salary</t>
+  </si>
+  <si>
+    <t>felony</t>
+  </si>
+  <si>
+    <t>driver's license</t>
+  </si>
+  <si>
+    <t>Desired Pay</t>
+  </si>
+  <si>
+    <t>highest degree</t>
+  </si>
+  <si>
+    <t>Bachelors Degree in Computer Science</t>
+  </si>
+  <si>
+    <t>certifications do you have</t>
+  </si>
+  <si>
+    <t>not applicable</t>
+  </si>
+  <si>
+    <t>current clearance</t>
+  </si>
+  <si>
+    <t>DHS Public Trust</t>
+  </si>
+  <si>
+    <t>preferred contact method</t>
+  </si>
+  <si>
+    <t>Phone, anytime.</t>
   </si>
 </sst>
 </file>
@@ -615,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.42578125" customWidth="1"/>
@@ -636,76 +669,76 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
         <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -713,54 +746,54 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
         <v>12</v>
-      </c>
-      <c r="C9" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
         <v>15</v>
-      </c>
-      <c r="C10" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -768,32 +801,32 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C16">
         <v>5</v>
@@ -801,10 +834,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C17">
         <v>4</v>
@@ -812,10 +845,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -823,10 +856,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -834,54 +867,54 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C21" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B22" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -889,10 +922,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B25" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C25">
         <v>4</v>
@@ -900,10 +933,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -911,10 +944,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B27" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C27">
         <v>4</v>
@@ -922,10 +955,10 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C28">
         <v>120000</v>
@@ -933,142 +966,142 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C29" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B30" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C30" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B31" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C31" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B32" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C32" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B33" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C33" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B34" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C34" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B35" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C35" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B36" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C36" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B37" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C37" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B38" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C38" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C39" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B40" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C40" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C41">
         <v>120000</v>
@@ -1076,65 +1109,65 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B42" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C42" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B43" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C43" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B44" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C44" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B45" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C45" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B46" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C46" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B47" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C47">
         <v>3</v>
@@ -1142,10 +1175,10 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B48" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C48">
         <v>4</v>
@@ -1153,134 +1186,211 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B49" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C49" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B50" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C50" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B51" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C51" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B52" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C52" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B53" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C53" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B54" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C54" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B55" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C55" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B56" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C56" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B57" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C57" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B58" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C58" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B59" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C59" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B60" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C60">
         <v>6</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>85</v>
+      </c>
+      <c r="B61" t="s">
+        <v>7</v>
+      </c>
+      <c r="C61" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>86</v>
+      </c>
+      <c r="B62" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>87</v>
+      </c>
+      <c r="B63" t="s">
+        <v>10</v>
+      </c>
+      <c r="C63">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>88</v>
+      </c>
+      <c r="B64" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>90</v>
+      </c>
+      <c r="B65" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>92</v>
+      </c>
+      <c r="B66" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67" t="s">
+        <v>10</v>
+      </c>
+      <c r="C67" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finished implementing the write to excel after taking in the Question, Type, Value infomration from the Window gui
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -1,28 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4507"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="390" yWindow="525" windowWidth="15015" windowHeight="11445"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$29</definedName>
-  </definedNames>
   <calcPr calcId="125725"/>
-  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="95">
   <si>
     <t>Question</t>
   </si>
@@ -33,6 +25,18 @@
     <t>Value</t>
   </si>
   <si>
+    <t>US Citizen</t>
+  </si>
+  <si>
+    <t>radio</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>u.s. citizen</t>
+  </si>
+  <si>
     <t>Do you have a Bachelor's Degree</t>
   </si>
   <si>
@@ -45,12 +49,6 @@
     <t>receiving text communications</t>
   </si>
   <si>
-    <t>radio</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
     <t>years of ServiceNow experience</t>
   </si>
   <si>
@@ -63,12 +61,12 @@
     <t>no, I have a DHS Public Trust</t>
   </si>
   <si>
+    <t>Day</t>
+  </si>
+  <si>
     <t>select-one</t>
   </si>
   <si>
-    <t>Day</t>
-  </si>
-  <si>
     <t>Weekday</t>
   </si>
   <si>
@@ -78,57 +76,57 @@
     <t>Anytime (8am - 9pm)</t>
   </si>
   <si>
+    <t>able to relocate</t>
+  </si>
+  <si>
+    <t>Doesn't apply</t>
+  </si>
+  <si>
+    <t>How many years of Robotic Process Automation</t>
+  </si>
+  <si>
+    <t>Describe your experience with UiPath or similar technologies</t>
+  </si>
+  <si>
+    <t>While I haven’t used UiPath directly, I have hands-on experience building automation workflows using Python and scripting tools to perform tasks similar to what UiPath enables. At MobileFrontiers, I wrote automation scripts for containerized environments using Docker, streamlining repetitive setup and deployment processes. In another project, I developed a Python-based GUI tool using Selenium, Tkinter, and pandas to automate web form submissions, data extraction, and Excel integration — all user-controlled through a front-end interface. These solutions handled decision logic, error handling, and multi-step workflows, closely aligning with the goals of RPA tools like UiPath. I’m confident I can apply these skills to UiPath or similar platforms with minimal ramp-up time.</t>
+  </si>
+  <si>
+    <t>position requires US citizenship</t>
+  </si>
+  <si>
+    <t>Yes- and I have a DHS Public Trust</t>
+  </si>
+  <si>
+    <t>How many years of Java experience do you have?</t>
+  </si>
+  <si>
+    <t>How many years of AWS experience do you have?</t>
+  </si>
+  <si>
+    <t>How many years of Microservices experience do you have?</t>
+  </si>
+  <si>
+    <t>How many years of MongoDB experience do you have?</t>
+  </si>
+  <si>
+    <t>required citizenship status is US Citizen</t>
+  </si>
+  <si>
+    <t>Apply anyway</t>
+  </si>
+  <si>
     <t>button</t>
   </si>
   <si>
+    <t>When are you available to start</t>
+  </si>
+  <si>
+    <t>Anytime</t>
+  </si>
+  <si>
     <t>Continue</t>
   </si>
   <si>
-    <t>able to relocate</t>
-  </si>
-  <si>
-    <t>Doesn't apply</t>
-  </si>
-  <si>
-    <t>How many years of Robotic Process Automation</t>
-  </si>
-  <si>
-    <t>While I haven’t used UiPath directly, I have hands-on experience building automation workflows using Python and scripting tools to perform tasks similar to what UiPath enables. At MobileFrontiers, I wrote automation scripts for containerized environments using Docker, streamlining repetitive setup and deployment processes. In another project, I developed a Python-based GUI tool using Selenium, Tkinter, and pandas to automate web form submissions, data extraction, and Excel integration — all user-controlled through a front-end interface. These solutions handled decision logic, error handling, and multi-step workflows, closely aligning with the goals of RPA tools like UiPath. I’m confident I can apply these skills to UiPath or similar platforms with minimal ramp-up time.</t>
-  </si>
-  <si>
-    <t>Describe your experience with UiPath or similar technologies</t>
-  </si>
-  <si>
-    <t>position requires US citizenship</t>
-  </si>
-  <si>
-    <t>Yes- and I have a DHS Public Trust</t>
-  </si>
-  <si>
-    <t>How many years of Java experience do you have?</t>
-  </si>
-  <si>
-    <t>How many years of AWS experience do you have?</t>
-  </si>
-  <si>
-    <t>How many years of Microservices experience do you have?</t>
-  </si>
-  <si>
-    <t>How many years of MongoDB experience do you have?</t>
-  </si>
-  <si>
-    <t>required citizenship status is US Citizen</t>
-  </si>
-  <si>
-    <t>Apply anyway</t>
-  </si>
-  <si>
-    <t>When are you available to start</t>
-  </si>
-  <si>
-    <t>Anytime</t>
-  </si>
-  <si>
     <t>How many years of HP Non Stop / Tandem experience do you have?</t>
   </si>
   <si>
@@ -141,6 +139,9 @@
     <t>How many years of applicable experience do you have?</t>
   </si>
   <si>
+    <t>salary</t>
+  </si>
+  <si>
     <t>Do you have a TS/SCI with CI poly?</t>
   </si>
   <si>
@@ -231,9 +232,6 @@
     <t>Clearance Level</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>Gender</t>
   </si>
   <si>
@@ -268,15 +266,6 @@
   </si>
   <si>
     <t>How many years of modern JavaScript experience do you have?</t>
-  </si>
-  <si>
-    <t>US Citizen</t>
-  </si>
-  <si>
-    <t>u.s. citizen</t>
-  </si>
-  <si>
-    <t>salary</t>
   </si>
   <si>
     <t>felony</t>
@@ -316,7 +305,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -324,34 +313,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -359,29 +335,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
@@ -396,44 +379,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -460,15 +443,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -495,7 +477,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -507,142 +488,166 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -651,16 +656,14 @@
   <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="42.42578125" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" customWidth="1"/>
-    <col min="3" max="3" width="53.85546875" customWidth="1"/>
+    <col min="1" max="1" width="36.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -669,76 +672,76 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
         <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -746,35 +749,35 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" t="s">
-        <v>13</v>
-      </c>
       <c r="C11" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -782,7 +785,7 @@
         <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C12" t="s">
         <v>21</v>
@@ -793,7 +796,7 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -801,13 +804,13 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
         <v>24</v>
-      </c>
-      <c r="B14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -815,7 +818,7 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
         <v>26</v>
@@ -826,7 +829,7 @@
         <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C16">
         <v>5</v>
@@ -837,7 +840,7 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C17">
         <v>4</v>
@@ -848,7 +851,7 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -859,7 +862,7 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -870,7 +873,7 @@
         <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C20" t="s">
         <v>26</v>
@@ -881,7 +884,7 @@
         <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="C21" t="s">
         <v>32</v>
@@ -889,32 +892,32 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="B23" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="C23" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B24" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -922,10 +925,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B25" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C25">
         <v>4</v>
@@ -933,10 +936,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -944,10 +947,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B27" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C27">
         <v>4</v>
@@ -955,10 +958,10 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="B28" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C28">
         <v>120000</v>
@@ -966,142 +969,142 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B29" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B30" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B31" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C31" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
         <v>43</v>
-      </c>
-      <c r="B32" t="s">
-        <v>7</v>
-      </c>
-      <c r="C32" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B33" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B34" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B35" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B36" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B37" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C37" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B38" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B39" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B40" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C40" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B41" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C41">
         <v>120000</v>
@@ -1109,65 +1112,65 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B42" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C42" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B43" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C43" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B44" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C44" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B45" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B46" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B47" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C47">
         <v>3</v>
@@ -1175,10 +1178,10 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B48" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C48">
         <v>4</v>
@@ -1186,131 +1189,128 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B49" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C49" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B50" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B51" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B52" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C52" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B53" t="s">
-        <v>7</v>
-      </c>
-      <c r="C53" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B54" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C54" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B55" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C55" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B56" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B57" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C57" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B58" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C58" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B59" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B60" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C60">
         <v>6</v>
@@ -1318,32 +1318,32 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B61" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C61" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B62" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C62" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B63" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C63">
         <v>120000</v>
@@ -1351,62 +1351,49 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
+        <v>87</v>
+      </c>
+      <c r="B64" t="s">
+        <v>12</v>
+      </c>
+      <c r="C64" t="s">
         <v>88</v>
-      </c>
-      <c r="B64" t="s">
-        <v>10</v>
-      </c>
-      <c r="C64" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
+        <v>89</v>
+      </c>
+      <c r="B65" t="s">
+        <v>12</v>
+      </c>
+      <c r="C65" t="s">
         <v>90</v>
-      </c>
-      <c r="B65" t="s">
-        <v>10</v>
-      </c>
-      <c r="C65" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
+        <v>91</v>
+      </c>
+      <c r="B66" t="s">
+        <v>12</v>
+      </c>
+      <c r="C66" t="s">
         <v>92</v>
-      </c>
-      <c r="B66" t="s">
-        <v>10</v>
-      </c>
-      <c r="C66" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
+        <v>93</v>
+      </c>
+      <c r="B67" t="s">
+        <v>12</v>
+      </c>
+      <c r="C67" t="s">
         <v>94</v>
       </c>
-      <c r="B67" t="s">
-        <v>10</v>
-      </c>
-      <c r="C67" t="s">
-        <v>95</v>
-      </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation errorStyle="information" allowBlank="1" showInputMessage="1" sqref="A23"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B10 B12:B23 B25:B1048576">
-      <formula1>"radio, select, text, select-one, button"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="information" allowBlank="1" showInputMessage="1" sqref="C1:C23 C25:C1048576">
-      <formula1>"yes, no"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11">
-      <formula1>"radio, select, text, select-one"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed a few bugs, main one was making sure that window object's combo_QTV instance attribute was updated after writing new excel entry in excel_QTV
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1667,6 +1667,24 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">middle name
+</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>uz</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
1) Added copy and paste feature for textarea_handling using pyperclip, efficient and fast for long strings 2) fixed bug- instead of a equality for radio button, I switched to checking if value is a partial string with in.
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,71 +499,75 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> requires a minimum of three(3) years of physical presence in the U.S.</t>
+          <t>which agency granted your clearance or public trust (e.g., dod, doe, fbi, nasa)?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>DHS</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>How many years of HP Non Stop / Tandem experience do you have?</t>
+          <t xml:space="preserve"> requires a minimum of three(3) years of physical presence in the U.S.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>How many years of Linux Administration experience do you have?</t>
+          <t>how many years of experience do you have in a similar type of role?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>3</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Describe your experience with UiPath or similar technologies</t>
+          <t>do you have at least 5 years of experience with peoplesoft hcm?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>While I haven’t used UiPath directly, I have hands-on experience building automation workflows using Python and scripting tools to perform tasks similar to what UiPath enables. At MobileFrontiers, I wrote automation scripts for containerized environments using Docker, streamlining repetitive setup and deployment processes. In another project, I developed a Python-based GUI tool using Selenium, Tkinter, and pandas to automate web form submissions, data extraction, and Excel integration — all user-controlled through a front-end interface. These solutions handled decision logic, error handling, and multi-step workflows, closely aligning with the goals of RPA tools like UiPath. I’m confident I can apply these skills to UiPath or similar platforms with minimal ramp-up time.</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>How many years of modern JavaScript experience do you have?</t>
+          <t>How many years of Linux Administration experience do you have?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -572,13 +576,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>How many years of Microservices experience do you have?</t>
+          <t>How many years of HP Non Stop / Tandem experience do you have?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -587,47 +591,45 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Do you have 1 or more of the following certifications?</t>
+          <t>Describe your experience with UiPath or similar technologies</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>While I haven’t used UiPath directly, I have hands-on experience building automation workflows using Python and scripting tools to perform tasks similar to what UiPath enables. At MobileFrontiers, I wrote automation scripts for containerized environments using Docker, streamlining repetitive setup and deployment processes. In another project, I developed a Python-based GUI tool using Selenium, Tkinter, and pandas to automate web form submissions, data extraction, and Excel integration — all user-controlled through a front-end interface. These solutions handled decision logic, error handling, and multi-step workflows, closely aligning with the goals of RPA tools like UiPath. I’m confident I can apply these skills to UiPath or similar platforms with minimal ramp-up time.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>require any immigration related support or sponsorship</t>
+          <t>How many years of modern JavaScript experience do you have?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Do you currently have a relative or spouse working at</t>
+          <t>do you have an active ts/sci clearance and fs polygraph? *</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -644,69 +646,73 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Do you have an active Top Secret security clearance?</t>
+          <t>How many years of Microservices experience do you have?</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>How many years of applicable experience do you have?</t>
+          <t>require any immigration related support or sponsorship</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>applied DevOps professional experience do you have?</t>
+          <t>Do you have 1 or more of the following certifications?</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>How many years of airflow experience do you have?</t>
+          <t>Do you currently have a relative or spouse working at</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>How many years of MongoDB experience do you have?</t>
+          <t>How many years of applicable experience do you have?</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -715,79 +721,78 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>How many years of Python experience do you have?</t>
+          <t>do you want to tell us anything else about yourself?</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>4</v>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Automated Job Application Tool – Personal Project | May 2025 – Present
+Developed a Python desktop automation tool using Selenium, Tkinter, and pandas to auto-fill online job applications. Designed a GUI to control flow and dynamically update form data from Excel files. Implemented DOM scraping and fuzzy string matching to identify and interact with visible form elements (textboxes, radio buttons, dropdowns). Enabled Chrome remote debugging for resilient, real-time automation and built intelligent logic to skip irrelevant pages and adapt behavior based on the page URL. Link: github.com/RaqibZaman/AutomateJobApplication</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Please list any relevant certifications you hold</t>
+          <t>Do you have an active Top Secret security clearance?</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Do you have 5+ years of Microsoft Power Platform</t>
+          <t>applied DevOps professional experience do you have?</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Do you have 8+ years of Microsoft Power Platform</t>
+          <t>How many years of MongoDB experience do you have?</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Are you eligible to work in the United States?</t>
+          <t>lived in the us for at least the last three years</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -804,7 +809,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>How many years of Java experience do you have?</t>
+          <t>How many years of airflow experience do you have?</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -813,60 +818,62 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>How many years of AWS experience do you have?</t>
+          <t>by submitting your application you hereby certify</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Are you able to obtain a Government Clearance</t>
+          <t>How many years of Python experience do you have?</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>How many years of Robotic Process Automation</t>
+          <t>Do you have 8+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>2</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>high school/university/college degrees held</t>
+          <t>Please list any relevant certifications you hold</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -876,48 +883,46 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Bachelor's in Computer Science</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>required citizenship status is US Citizen</t>
+          <t>Do you have 5+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Yes- and I have a DHS Public Trust</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>participate in any stage of a procurement</t>
+          <t>How many years of Java experience do you have?</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>authorized to work in the United States</t>
+          <t>Are you eligible to work in the United States?</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -934,54 +939,54 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>active and relevant certifications held</t>
+          <t>Are you able to obtain a Government Clearance</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Are you authorized to work in the US?</t>
+          <t>How many years of AWS experience do you have?</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Have you previously been employed by</t>
+          <t>How many years of Robotic Process Automation</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Do you have the necessary experience</t>
+          <t>are you authorized to work in united states</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -991,31 +996,31 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>I am authorized to work in this country for any employer</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Will you be able to reliably commute</t>
+          <t>high school/university/college degrees held</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Bachelor's in Computer Science</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>is your clearance currently active?</t>
+          <t>submit a drug screen and background check?</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1032,56 +1037,58 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Do you hold an active TS/SCI w/FSP?</t>
+          <t>participate in any stage of a procurement</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>no, I have a DHS Public Trust</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Total years of relative experience?</t>
+          <t>required citizenship status is US Citizen</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2+</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>What are your salary expectations?</t>
+          <t>do you have us. gov't security clearance?</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>120000</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Do you have a valid US Citizenship</t>
+          <t>what type of employment are you seeking?</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1091,14 +1098,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>full time</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Do you have a TS/SCI with CI poly?</t>
+          <t>current position for at least 12 months?</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1108,39 +1115,441 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>years of relevant work experience</t>
+          <t>authorized to work in the United States</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>what is your annual salary requirement?</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>how did you hear about this position? *</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>active and relevant certifications held</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>when would you be able to start working</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Are you authorized to work in the US?</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>live in the united states of america?</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>What is your current location (State)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>virginia</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>current level of an active clearance?</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>DHS Public Trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>how did you hear about the position?</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Have you previously been employed by</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Will you be able to reliably commute</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>please select your disability status</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>I don't have a disability</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Do you have the necessary experience</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>highest level of education obtained?</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Do you hold an active TS/SCI w/FSP?</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>no, I have a DHS Public Trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Total years of relative experience?</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2+</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>is your clearance currently active?</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>eligible to obtain a public trust?</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Do you have a TS/SCI with CI poly?</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Do you have a valid US Citizenship</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>What are your salary expectations?</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>years of relevant work experience</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>please select your veteran status</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>I am not a protected veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>former employee of any government</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>never</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>please copy and paste your resume</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>textarea</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>Raqib Zaman
 Lorton, VA | 703-473-5140 | raqib.zaman@gmail.com LinkedIn: linkedin.com/in/raqibzaman 
@@ -1204,429 +1613,27 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>former employee of any government</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>never</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>position requires US citizenship</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Yes- and I have a DHS Public Trust</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>When are you available to start</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Anytime</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Do you have a Bachelor's Degree</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>years of ServiceNow experience</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Are you located in Arizona? *</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>receiving text communications</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>how did you hear about us? *</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Are you a protected Veteran?</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>certifications do you have</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>not applicable</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Protected Veteran Status</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>I am not a protected veteran</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>do you want to opt-in? *</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>require visa sponsorship</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>preferred contact method</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Phone, anytime.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>willing to relocate?</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>active DoD clearance</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>security clearance</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Public Trust</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>current clearance</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>DHS Public Trust</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>disability status</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Disability Status</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>No, I do not have a disability and have not had one in the past</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>select your race</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Asian</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>driver's license</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>able to relocate</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Doesn't apply</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Clearance Level</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr"/>
-    </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>veteran status</t>
+          <t>position requires US citizenship</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>not a protected veteran</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>we may use sms during the hiring</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1636,31 +1643,31 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>I am not a veteran</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>highest degree</t>
+          <t>have an active secret clearance?</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Bachelors Degree in Computer Science</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>date available</t>
+          <t>how did you hear about this job?</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1670,14 +1677,14 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>online search</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>u.s. citizen</t>
+          <t>Do you have a Bachelor's Degree</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1694,24 +1701,24 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>do you have federal experience?</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>middle name</t>
+          <t>When are you available to start</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1721,14 +1728,14 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>uz</t>
+          <t>Anytime</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Desired Pay</t>
+          <t>years of ServiceNow experience</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -1737,13 +1744,13 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>120000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>US Citizen</t>
+          <t>what is your desired salary? *</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -1753,14 +1760,14 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Annual</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Are you located in Arizona? *</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1770,137 +1777,879 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Bachelors Degree</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Continue</t>
+          <t>receiving text communications</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Continue</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>felony</t>
+          <t>please enter the amount ($) *</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>how did you hear about us? *</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Indeed</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>salary</t>
+          <t>Are you a protected Veteran?</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C82" t="n">
-        <v>120000</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>suffix</t>
+          <t>are you a military veteran?</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>require a visa sponsorship</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Anytime (8am - 9pm)</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Race</t>
+          <t>certifications do you have</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Asian</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>do you want to opt-in? *</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Protected Veteran Status</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>I am not a protected veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>preferred contact method</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Phone, anytime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>require visa sponsorship</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>require any sponsorship</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>best method to contact</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>desired compensation?</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>120000</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>if you were referred</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>active DoD clearance</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>willing to relocate?</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>require sponsorship</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>reside in the u.s.</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>security clearance</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Public Trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>level of education</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>4 Year University</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>disability status</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>current clearance</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>DHS Public Trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Disability Status</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>No, I do not have a disability and have not had one in the past</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>ts/sci with poly</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>select your race</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>able to relocate</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Doesn't apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>driver's license</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Clearance Level</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>veteran status</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>not a protected veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>date available</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>highest degree</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Bachelors Degree in Computer Science</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Veteran Status</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>I am not a veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>u.s. citizen</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Apply anyway</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Apply anyway</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>middle name</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>uz</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Desired Pay</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>US Citizen</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>disability</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Bachelors Degree</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>ethnicity</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Continue</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>felony</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>suffix</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Anytime (8am - 9pm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Raqib Zaman</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B129" t="inlineStr">
         <is>
           <t>select-one</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C129" t="inlineStr">
         <is>
           <t>Weekday</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>22079</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added a simple debug button if I want to pause execution in a certain part of my code, due to missing excel entry or otherwise
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1616,17 +1616,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>position requires US citizenship</t>
+          <t>do you have an irs mbi clearance?</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Yes- and I have a DHS Public Trust</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1650,17 +1650,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>have an active secret clearance?</t>
+          <t>position requires US citizenship</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Do you have a Bachelor's Degree</t>
+          <t>have an active secret clearance?</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1718,24 +1718,24 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>When are you available to start</t>
+          <t>Do you have a Bachelor's Degree</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Anytime</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>years of ServiceNow experience</t>
+          <t>When are you available to start</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -1743,31 +1743,31 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C76" t="n">
-        <v>1</v>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Anytime</t>
+        </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>what is your desired salary? *</t>
+          <t>years of ServiceNow experience</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Annual</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Are you located in Arizona? *</t>
+          <t>what is your desired salary? *</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1777,14 +1777,14 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Annual</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>receiving text communications</t>
+          <t>Are you located in Arizona? *</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1818,17 +1818,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>how did you hear about us? *</t>
+          <t>receiving text communications</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1852,24 +1852,24 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>are you a military veteran?</t>
+          <t>how did you hear about us? *</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Indeed</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>require a visa sponsorship</t>
+          <t>are you a military veteran?</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -1886,41 +1886,41 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>certifications do you have</t>
+          <t>require a visa sponsorship</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>do you want to opt-in? *</t>
+          <t>certifications do you have</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Protected Veteran Status</t>
+          <t>do you want to opt-in? *</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>I am not a protected veteran</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>require any sponsorship</t>
+          <t>Protected Veteran Status</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -1981,14 +1981,14 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>I am not a protected veteran</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>best method to contact</t>
+          <t>require any sponsorship</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -1998,41 +1998,41 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>desired compensation?</t>
+          <t>best method to contact</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>120000</t>
+          <t>email</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>if you were referred</t>
+          <t>desired compensation?</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
@@ -2056,24 +2056,24 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>willing to relocate?</t>
+          <t>if you were referred</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>require sponsorship</t>
+          <t>willing to relocate?</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2090,7 +2090,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>reside in the u.s.</t>
+          <t>require sponsorship</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2124,51 +2124,51 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>level of education</t>
+          <t>reside in the u.s.</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>4 Year University</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>disability status</t>
+          <t>level of education</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>4 Year University</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>current clearance</t>
+          <t>disability status</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2192,17 +2192,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ts/sci with poly</t>
+          <t>current clearance</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Clearance Level</t>
+          <t>ts/sci with poly</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2268,12 +2268,16 @@
           <t>radio</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>veteran status</t>
+          <t>Clearance Level</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2281,26 +2285,22 @@
           <t>radio</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>not a protected veteran</t>
-        </is>
-      </c>
+      <c r="C108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>date available</t>
+          <t>veteran status</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>not a protected veteran</t>
         </is>
       </c>
     </row>
@@ -2324,24 +2324,24 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>date available</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>I am not a veteran</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>u.s. citizen</t>
+          <t>Veteran Status</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2351,48 +2351,48 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>I am not a veteran</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>u.s. citizen</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>middle name</t>
+          <t>Apply anyway</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>button</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>uz</t>
+          <t>Apply anyway</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Desired Pay</t>
+          <t>middle name</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -2400,31 +2400,31 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C115" t="n">
-        <v>120000</v>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>uz</t>
+        </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>US Citizen</t>
+          <t>Desired Pay</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>disability</t>
+          <t>US Citizen</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -2434,14 +2434,14 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>disability</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2451,58 +2451,58 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Bachelors Degree</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ethnicity</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>asian</t>
+          <t>Bachelors Degree</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Continue</t>
+          <t>ethnicity</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Continue</t>
+          <t>asian</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Continue</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>button</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Continue</t>
         </is>
       </c>
     </row>
@@ -2526,20 +2526,24 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>suffix</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>salary</t>
+          <t>suffix</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -2547,25 +2551,21 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C124" t="n">
-        <v>120000</v>
-      </c>
+      <c r="C124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Race</t>
+          <t>salary</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Asian</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="126">
@@ -2588,24 +2588,24 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>Race</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Raqib Zaman</t>
+          <t>Asian</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -2615,39 +2615,56 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>Raqib Zaman</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Weekday</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Weekday</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
           <t>zip</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
         <is>
           <t>22079</t>
         </is>

</xml_diff>

<commit_message>
1) Customized appending node to array i.e. rank is elevanted from child to parent node if new_nod.tag == fieldset. 2) For select-one, I decided to loop through matched dataframe result rows for select-one, in select_handling 3) trying to handle special cases like entering in a cover letter and so on.
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,24 +533,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>how many years of experience do you have in a similar type of role?</t>
+          <t>if you were referred by a gunnison employee, please provide the name</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>Rahat Sultan</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>do you have at least 5 years of experience with peoplesoft hcm?</t>
+          <t>how many years of experience do you have in a similar type of role?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -560,44 +560,48 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>How many years of Linux Administration experience do you have?</t>
+          <t>please review the salary range for the position. would you accept</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>3</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>How many years of HP Non Stop / Tandem experience do you have?</t>
+          <t>do you have at least 5 years of experience with peoplesoft hcm?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Describe your experience with UiPath or similar technologies</t>
+          <t>How many years of HP Non Stop / Tandem experience do you have?</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -605,16 +609,14 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>While I haven’t used UiPath directly, I have hands-on experience building automation workflows using Python and scripting tools to perform tasks similar to what UiPath enables. At MobileFrontiers, I wrote automation scripts for containerized environments using Docker, streamlining repetitive setup and deployment processes. In another project, I developed a Python-based GUI tool using Selenium, Tkinter, and pandas to automate web form submissions, data extraction, and Excel integration — all user-controlled through a front-end interface. These solutions handled decision logic, error handling, and multi-step workflows, closely aligning with the goals of RPA tools like UiPath. I’m confident I can apply these skills to UiPath or similar platforms with minimal ramp-up time.</t>
-        </is>
+      <c r="C11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>How many years of modern JavaScript experience do you have?</t>
+          <t>How many years of Linux Administration experience do you have?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -623,13 +625,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>do you have an active ts/sci clearance and fs polygraph? *</t>
+          <t>would you be able and willing to travel as needed by the job?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -639,14 +641,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>How many years of Microservices experience do you have?</t>
+          <t>Describe your experience with UiPath or similar technologies</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -654,31 +656,31 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>1</v>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>While I haven’t used UiPath directly, I have hands-on experience building automation workflows using Python and scripting tools to perform tasks similar to what UiPath enables. At MobileFrontiers, I wrote automation scripts for containerized environments using Docker, streamlining repetitive setup and deployment processes. In another project, I developed a Python-based GUI tool using Selenium, Tkinter, and pandas to automate web form submissions, data extraction, and Excel integration — all user-controlled through a front-end interface. These solutions handled decision logic, error handling, and multi-step workflows, closely aligning with the goals of RPA tools like UiPath. I’m confident I can apply these skills to UiPath or similar platforms with minimal ramp-up time.</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>require any immigration related support or sponsorship</t>
+          <t>How many years of modern JavaScript experience do you have?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Do you have 1 or more of the following certifications?</t>
+          <t>are you able to perform the essential functions of the job</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -688,14 +690,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Do you currently have a relative or spouse working at</t>
+          <t>do you have an active ts/sci clearance and fs polygraph? *</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -712,151 +714,153 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>How many years of applicable experience do you have?</t>
+          <t>are you able to commute daily to the location indicated</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>How many years of Microservices experience do you have?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>if presently employed, why are you considering leaving?</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>require any immigration related support or sponsorship</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>if yes, please provide details (where/when/job title):</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Do you have 1 or more of the following certifications?</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Do you currently have a relative or spouse working at</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>How many years of applicable experience do you have?</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>do you want to tell us anything else about yourself?</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>textarea</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Automated Job Application Tool – Personal Project | May 2025 – Present
 Developed a Python desktop automation tool using Selenium, Tkinter, and pandas to auto-fill online job applications. Designed a GUI to control flow and dynamically update form data from Excel files. Implemented DOM scraping and fuzzy string matching to identify and interact with visible form elements (textboxes, radio buttons, dropdowns). Enabled Chrome remote debugging for resilient, real-time automation and built intelligent logic to skip irrelevant pages and adapt behavior based on the page URL. Link: github.com/RaqibZaman/AutomateJobApplication</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Do you have an active Top Secret security clearance?</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>applied DevOps professional experience do you have?</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>How many years of MongoDB experience do you have?</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>lived in the us for at least the last three years</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>How many years of airflow experience do you have?</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>by submitting your application you hereby certify</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>accept</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>How many years of Python experience do you have?</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>4</v>
-      </c>
-    </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Do you have 8+ years of Microsoft Power Platform</t>
+          <t>Do you have an active Top Secret security clearance?</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -873,7 +877,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Please list any relevant certifications you hold</t>
+          <t>applied DevOps professional experience do you have?</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -881,16 +885,14 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
+      <c r="C28" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Do you have 5+ years of Microsoft Power Platform</t>
+          <t>by submitting your application you hereby certify</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -900,14 +902,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>accept</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>How many years of Java experience do you have?</t>
+          <t>How many years of MongoDB experience do you have?</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -916,13 +918,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Are you eligible to work in the United States?</t>
+          <t>lived in the us for at least the last three years</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -939,105 +941,105 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Are you able to obtain a Government Clearance</t>
+          <t>How many years of airflow experience do you have?</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>How many years of AWS experience do you have?</t>
+          <t>Do you have 5+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>How many years of Robotic Process Automation</t>
+          <t>linux scripting language are you most proficient</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>2</v>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Bash, Python, and looking into Lua</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>are you authorized to work in united states</t>
+          <t>How many years of Python experience do you have?</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>I am authorized to work in this country for any employer</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>high school/university/college degrees held</t>
+          <t>Do you have 8+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Bachelor's in Computer Science</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>submit a drug screen and background check?</t>
+          <t>Please list any relevant certifications you hold</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>participate in any stage of a procurement</t>
+          <t>do you reside in one of the following us states</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1047,31 +1049,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>required citizenship status is US Citizen</t>
+          <t>please provide us with a copy of your agreement</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Yes- and I have a DHS Public Trust</t>
-        </is>
-      </c>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>do you have us. gov't security clearance?</t>
+          <t>Are you eligible to work in the United States?</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1088,41 +1086,37 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>what type of employment are you seeking?</t>
+          <t>How many years of Java experience do you have?</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>full time</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>current position for at least 12 months?</t>
+          <t>How many years of AWS experience do you have?</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>authorized to work in the United States</t>
+          <t>eligible to be employed in the united states?</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1139,41 +1133,41 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>what is your annual salary requirement?</t>
+          <t>Are you able to obtain a Government Clearance</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>how did you hear about this position? *</t>
+          <t>list the cloud providers you have experience</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>AWS, Azure, Digital Ocean</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>active and relevant certifications held</t>
+          <t>How many years of Robotic Process Automation</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1181,46 +1175,48 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>when would you be able to start working</t>
+          <t>are you authorized to work in united states</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>I am authorized to work in this country for any employer</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Are you authorized to work in the US?</t>
+          <t>high school/university/college degrees held</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Bachelor's in Computer Science</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>live in the united states of america?</t>
+          <t>submit a drug screen and background check?</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1237,58 +1233,58 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>What is your current location (State)</t>
+          <t>what is your availability to begin working</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>virginia</t>
+          <t>Anytime- Immediately.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>current level of an active clearance?</t>
+          <t>participate in any stage of a procurement</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>how did you hear about the position?</t>
+          <t>required citizenship status is US Citizen</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Have you previously been employed by</t>
+          <t>do you have us. gov't security clearance?</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1298,14 +1294,14 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Will you be able to reliably commute</t>
+          <t>what type of employment are you seeking?</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1315,14 +1311,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>full time</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>please select your disability status</t>
+          <t>may we inquire of your present employer?</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1332,14 +1328,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>I don't have a disability</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Do you have the necessary experience</t>
+          <t>current position for at least 12 months?</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1356,24 +1352,24 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>highest level of education obtained?</t>
+          <t>authorized to work in the United States</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Bachelor</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Do you hold an active TS/SCI w/FSP?</t>
+          <t>active and relevant certifications held</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1381,50 +1377,46 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>no, I have a DHS Public Trust</t>
-        </is>
-      </c>
+      <c r="C58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Total years of relative experience?</t>
+          <t>what is your annual salary requirement?</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2+</t>
+          <t>120</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>is your clearance currently active?</t>
+          <t>when would you be able to start working</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>eligible to obtain a public trust?</t>
+          <t>how did you hear about this position? *</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1434,14 +1426,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>other</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Do you have a TS/SCI with CI poly?</t>
+          <t>i have not entered into any non-compet</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1451,46 +1443,48 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Do you have a valid US Citizenship</t>
+          <t>how many years of relevant experience</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>4-5</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>What are your salary expectations?</t>
+          <t>live in the united states of america?</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>120000</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>years of relevant work experience</t>
+          <t>years of linux programming experience</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1507,24 +1501,24 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>please select your veteran status</t>
+          <t>security clearance you currently hold</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>I am not a protected veteran</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>former employee of any government</t>
+          <t>Are you authorized to work in the US?</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1534,22 +1528,360 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>never</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>current level of an active clearance?</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>DHS Public Trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>What is your current location (State)</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>virginia</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>how did you hear about the position?</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Do you have the necessary experience</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Will you be able to reliably commute</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Have you previously been employed by</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>please select your disability status</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>I don't have a disability</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>highest level of education obtained?</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>when would you be available to begin</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Total years of relative experience?</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2+</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Do you hold an active TS/SCI w/FSP?</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>no, I have a DHS Public Trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>is your clearance currently active?</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>eligible to obtain a public trust?</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>What are your salary expectations?</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Do you have a TS/SCI with CI poly?</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Do you have a valid US Citizenship</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>years of relevant work experience</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>former employee of any government</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>never</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>please select your veteran status</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>I am not a protected veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>please provide an non voip number</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>703-473-5140</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
           <t>please copy and paste your resume</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>textarea</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>Raqib Zaman
 Lorton, VA | 703-473-5140 | raqib.zaman@gmail.com LinkedIn: linkedin.com/in/raqibzaman 
@@ -1613,348 +1945,10 @@
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>do you have an irs mbi clearance?</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>we may use sms during the hiring</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>position requires US citizenship</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Yes- and I have a DHS Public Trust</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>how did you hear about this job?</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>online search</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>have an active secret clearance?</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>do you have federal experience?</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Do you have a Bachelor's Degree</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>When are you available to start</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Anytime</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>years of ServiceNow experience</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C77" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>what is your desired salary? *</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Annual</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Are you located in Arizona? *</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>please enter the amount ($) *</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>120000</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>receiving text communications</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Are you a protected Veteran?</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>how did you hear about us? *</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>are you a military veteran?</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>require a visa sponsorship</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>certifications do you have</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>not applicable</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>do you want to opt-in? *</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>preferred contact method</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Phone, anytime.</t>
-        </is>
-      </c>
-    </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>require visa sponsorship</t>
+          <t>do you have an irs mbi clearance?</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -1971,24 +1965,24 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Protected Veteran Status</t>
+          <t>how did you hear about this job?</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>I am not a protected veteran</t>
+          <t>online search</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>require any sponsorship</t>
+          <t>we may use sms during the hiring</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -1998,14 +1992,14 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>best method to contact</t>
+          <t>have an active secret clearance?</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2015,14 +2009,14 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>desired compensation?</t>
+          <t>position requires US citizenship</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2032,14 +2026,14 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>120000</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>active DoD clearance</t>
+          <t>worked for this company before?</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2056,24 +2050,24 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>if you were referred</t>
+          <t>When are you available to start</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>Anytime</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>willing to relocate?</t>
+          <t>Do you have a Bachelor's Degree</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2083,14 +2077,14 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>require sponsorship</t>
+          <t>do you have federal experience?</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2100,31 +2094,29 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>security clearance</t>
+          <t>years of ServiceNow experience</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Public Trust</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>reside in the u.s.</t>
+          <t>what is your desired salary? *</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2134,48 +2126,48 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Annual</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>level of education</t>
+          <t>receiving text communications</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>4 Year University</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>disability status</t>
+          <t>please enter the amount ($) *</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Disability Status</t>
+          <t>Are you located in Arizona? *</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2185,31 +2177,31 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>No, I do not have a disability and have not had one in the past</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>current clearance</t>
+          <t>Are you a protected Veteran?</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>select your race</t>
+          <t>how did you hear about us? *</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2219,14 +2211,14 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Asian</t>
+          <t>Indeed</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>able to relocate</t>
+          <t>are you a military veteran?</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2236,14 +2228,14 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Doesn't apply</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>driver's license</t>
+          <t>are you currently employed?</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2253,14 +2245,14 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ts/sci with poly</t>
+          <t>type of employment desired</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2270,14 +2262,14 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>full-time</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Clearance Level</t>
+          <t>require a visa sponsorship</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2285,46 +2277,50 @@
           <t>radio</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>veteran status</t>
+          <t>certifications do you have</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>not a protected veteran</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>highest degree</t>
+          <t>will you be able to start</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Bachelors Degree in Computer Science</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>date available</t>
+          <t>preferred contact method</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2334,14 +2330,14 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>Phone, anytime.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>Protected Veteran Status</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2351,14 +2347,14 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>I am not a veteran</t>
+          <t>I am not a protected veteran</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>u.s. citizen</t>
+          <t>do you want to opt-in? *</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2375,24 +2371,24 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>require visa sponsorship</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>middle name</t>
+          <t>professional references</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -2402,29 +2398,31 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>uz</t>
+          <t>Bunmi Toye: (443)-929-3603, John Garber: john.d.garber@gmail.com 575-649-0811, Nicole Jacobs: (703)-801-3421, Sejal Dhawan: sejaldhawan98@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Desired Pay</t>
+          <t>review your application</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C116" t="n">
-        <v>120000</v>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>review your application</t>
+        </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>US Citizen</t>
+          <t>require any sponsorship</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -2434,14 +2432,14 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>disability</t>
+          <t>best method to contact</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2451,14 +2449,14 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>email</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>able to work remotely</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -2468,48 +2466,48 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Bachelors Degree</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ethnicity</t>
+          <t>desired compensation?</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>asian</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Continue</t>
+          <t>if you were referred</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Continue</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>felony</t>
+          <t>active DoD clearance</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -2526,7 +2524,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>willing to relocate?</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -2536,42 +2534,48 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>suffix</t>
+          <t>require sponsorship</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>salary</t>
+          <t>reside in the u.s.</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C125" t="n">
-        <v>120000</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>security clearance</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -2581,14 +2585,14 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Anytime (8am - 9pm)</t>
+          <t>Public Trust</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Race</t>
+          <t>level of education</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -2598,14 +2602,14 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Asian</t>
+          <t>4 Year University</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>current clearance</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -2615,56 +2619,578 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Raqib Zaman</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>disability status</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Disability Status</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Weekday</t>
+          <t>No, I do not have a disability and have not had one in the past</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
+          <t>18 years or older</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>able to relocate</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Doesn't apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>ts/sci with poly</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>select your race</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>driver's license</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Clearance Level</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>date available</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>highest degree</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Bachelors Degree in Computer Science</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>veteran status</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>not a protected veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Veteran Status</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>I am not a veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>veteran status</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>not a veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>u.s. citizen</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Apply anyway</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Apply anyway</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>cover letter</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>enter text</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>middle name</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>uz</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Desired Pay</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>US Citizen</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>disability</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>enter text</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>[cover letter]</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Dear Hiring Manager,
+I am writing to express my interest in the Software Developer position at [Company Name], as advertised. With over four years of hands-on experience developing full stack enterprise web applications for federal clients, I bring a strong foundation in ASP.NET MVC, C#, JavaScript, SQL, and accessibility standards. My technical proficiency and dedication to delivering high-quality, compliant software solutions align well with your team’s mission.
+At Customer Value Partners (CVP), I have worked extensively on Department of Homeland Security (DHS) systems such as the Environmental Planning &amp; Historic Preservation Decision Support System (EPHP DSS) and the Federal Protective Service Post Tracking System (FPS PTS). In these roles, I designed and implemented complex reporting modules, dynamic form logic, and accessibility enhancements using C#, Entity Framework, JavaScript, and Oracle SQL. I’ve developed features like PDF/Excel export functionality, dynamic CATEX classification interfaces, and Section 508/WCAG 2.0 compliance upgrades—directly improving efficiency and usability for government users.
+In addition to full stack development, I bring experience in DevOps automation through my internship at Mobile Frontiers, where I built tools using Python, Docker, and AWS SDK (boto3) to support satellite communications and cloud resource optimization. I also recently built a personal job automation tool using Selenium and Tkinter, which demonstrates my initiative, problem-solving mindset, and versatility with automation and UI frameworks.
+I hold a Bachelor’s degree in Computer Science from George Mason University and maintain Public Trust clearance. My passion lies in building intuitive, accessible, and robust applications that not only meet functional requirements but also serve diverse users effectively.
+I would welcome the opportunity to discuss how my background and skill set can contribute to your team. Thank you for considering my application. I am available at your convenience for an interview and can be reached at raqib.zaman@gmail.com or 703-473-5140.
+Sincerely,
+Raqib Zaman</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Bachelors Degree</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>ethnicity</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Continue</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>felony</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>suffix</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Anytime (8am - 9pm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Raqib Zaman</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Weekday</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
           <t>zip</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
         <is>
           <t>22079</t>
         </is>

</xml_diff>

<commit_message>
So now I am looping through the whole set of matches, as I should have done in the beginning. For chunking the data, I should record the fieldset depth and perhaps 'assign' that to the legend in some way? Still not sure whats the best solution there- I should have started with a recursive tree solution from the get go, oh well. Pages differ too much so its hard to be consistent after updating the note array algorithm
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C162"/>
+  <dimension ref="A1:C208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,24 +448,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Are you able to perform the functions of the job, with or without reasonable accomodations?</t>
+          <t>Authorization: By entering your name below, you are verifying that you have read and understand the disclaimer below</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Raqib Zaman</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Do you need, or will you need in the future, any immigration-related support or sponsorship</t>
+          <t>Are you able to perform the functions of the job, with or without reasonable accomodations?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -475,31 +475,31 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Do you have an active government clearance? Please list specifics in the text field</t>
+          <t>Do you need, or will you need in the future, any immigration-related support or sponsorship</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yes, DHS Public Trust</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>which agency granted your clearance or public trust (e.g., dod, doe, fbi, nasa)?</t>
+          <t>Do you have an active government clearance? Please list specifics in the text field</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -509,14 +509,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DHS</t>
+          <t>Yes, DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> requires a minimum of three(3) years of physical presence in the U.S.</t>
+          <t>do you have experience designing, implementing, and maintaining aws-based solutions</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -533,7 +533,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>if you were referred by a gunnison employee, please provide the name</t>
+          <t>which agency granted your clearance or public trust (e.g., dod, doe, fbi, nasa)?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -543,14 +543,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Rahat Sultan</t>
+          <t>DHS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>how many years of experience do you have in a similar type of role?</t>
+          <t xml:space="preserve"> requires a minimum of three(3) years of physical presence in the U.S.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -560,31 +560,31 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>please review the salary range for the position. would you accept</t>
+          <t>if you were referred by a gunnison employee, please provide the name</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Rahat Sultan</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>do you have at least 5 years of experience with peoplesoft hcm?</t>
+          <t>how many years of experience do you have in a similar type of role?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -594,61 +594,63 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>How many years of HP Non Stop / Tandem experience do you have?</t>
+          <t>please review the salary range for the position. would you accept</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>How many years of Linux Administration experience do you have?</t>
+          <t>do you have at least 5 years of experience with peoplesoft hcm?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>3</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>would you be able and willing to travel as needed by the job?</t>
+          <t>How many years of HP Non Stop / Tandem experience do you have?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Describe your experience with UiPath or similar technologies</t>
+          <t>How many years of Linux Administration experience do you have?</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -656,65 +658,63 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>While I haven’t used UiPath directly, I have hands-on experience building automation workflows using Python and scripting tools to perform tasks similar to what UiPath enables. At MobileFrontiers, I wrote automation scripts for containerized environments using Docker, streamlining repetitive setup and deployment processes. In another project, I developed a Python-based GUI tool using Selenium, Tkinter, and pandas to automate web form submissions, data extraction, and Excel integration — all user-controlled through a front-end interface. These solutions handled decision logic, error handling, and multi-step workflows, closely aligning with the goals of RPA tools like UiPath. I’m confident I can apply these skills to UiPath or similar platforms with minimal ramp-up time.</t>
-        </is>
+      <c r="C14" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>How many years of modern JavaScript experience do you have?</t>
+          <t>would you be able and willing to travel as needed by the job?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>6</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>are you able to perform the essential functions of the job</t>
+          <t>Describe your experience with UiPath or similar technologies</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>While I haven’t used UiPath directly, I have hands-on experience building automation workflows using Python and scripting tools to perform tasks similar to what UiPath enables. At MobileFrontiers, I wrote automation scripts for containerized environments using Docker, streamlining repetitive setup and deployment processes. In another project, I developed a Python-based GUI tool using Selenium, Tkinter, and pandas to automate web form submissions, data extraction, and Excel integration — all user-controlled through a front-end interface. These solutions handled decision logic, error handling, and multi-step workflows, closely aligning with the goals of RPA tools like UiPath. I’m confident I can apply these skills to UiPath or similar platforms with minimal ramp-up time.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>do you have an active ts/sci clearance and fs polygraph? *</t>
+          <t>How many years of modern JavaScript experience do you have?</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>are you able to commute daily to the location indicated</t>
+          <t>are you able to perform the essential functions of the job</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -731,86 +731,90 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>How many years of Microservices experience do you have?</t>
+          <t>do you have an active ts/sci clearance and fs polygraph? *</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>1</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>if presently employed, why are you considering leaving?</t>
+          <t>experience with code vulnerability mitigation/remediation</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>require any immigration related support or sponsorship</t>
+          <t>How many years of Microservices experience do you have?</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>if yes, please provide details (where/when/job title):</t>
+          <t>are you able to commute daily to the location indicated</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Do you have 1 or more of the following certifications?</t>
+          <t>if presently employed, why are you considering leaving?</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Do you currently have a relative or spouse working at</t>
+          <t>require any immigration related support or sponsorship</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -827,104 +831,104 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>How many years of applicable experience do you have?</t>
+          <t>Do you have 1 or more of the following certifications?</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>if yes, please provide details (where/when/job title):</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>duties or responsibilities on behalf of the government</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Do you currently have a relative or spouse working at</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>How many years of applicable experience do you have?</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>do you want to tell us anything else about yourself?</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>textarea</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Automated Job Application Tool – Personal Project | May 2025 – Present
 Developed a Python desktop automation tool using Selenium, Tkinter, and pandas to auto-fill online job applications. Designed a GUI to control flow and dynamically update form data from Excel files. Implemented DOM scraping and fuzzy string matching to identify and interact with visible form elements (textboxes, radio buttons, dropdowns). Enabled Chrome remote debugging for resilient, real-time automation and built intelligent logic to skip irrelevant pages and adapt behavior based on the page URL. Link: github.com/RaqibZaman/AutomateJobApplication</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Do you have an active Top Secret security clearance?</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>applied DevOps professional experience do you have?</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>by submitting your application you hereby certify</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>accept</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>How many years of MongoDB experience do you have?</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
-    </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>lived in the us for at least the last three years</t>
+          <t>Do you have an active Top Secret security clearance?</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -934,14 +938,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>How many years of airflow experience do you have?</t>
+          <t>applied DevOps professional experience do you have?</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -950,13 +954,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Do you have 5+ years of Microsoft Power Platform</t>
+          <t>by submitting your application you hereby certify</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -966,31 +970,29 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>accept</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>linux scripting language are you most proficient</t>
+          <t>How many years of MongoDB experience do you have?</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>textarea</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Bash, Python, and looking into Lua</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>How many years of Python experience do you have?</t>
+          <t>How many years of airflow experience do you have?</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -999,13 +1001,13 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Do you have 8+ years of Microsoft Power Platform</t>
+          <t>lived in the us for at least the last three years</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1015,78 +1017,80 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Please list any relevant certifications you hold</t>
+          <t>Do you have 5+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>do you reside in one of the following us states</t>
+          <t>linux scripting language are you most proficient</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Bash, Python, and looking into Lua</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>please provide us with a copy of your agreement</t>
+          <t>Do you have 8+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>button</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Are you eligible to work in the United States?</t>
+          <t>How many years of Python experience do you have?</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>How many years of Java experience do you have?</t>
+          <t>Please list any relevant certifications you hold</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1094,95 +1098,95 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C41" t="n">
-        <v>5</v>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>How many years of AWS experience do you have?</t>
+          <t>do you reside in one of the following us states</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>eligible to be employed in the united states?</t>
+          <t>please provide us with a copy of your agreement</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Are you able to obtain a Government Clearance</t>
+          <t>Confirm Home Address (Street, City, State, Zip)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>8324 Middle Ruddings Dr, Lorton, VA, 22079</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>list the cloud providers you have experience</t>
+          <t>How many years of Java experience do you have?</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>textarea</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>AWS, Azure, Digital Ocean</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>How many years of Robotic Process Automation</t>
+          <t>Are you eligible to work in the United States?</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>2</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>are you authorized to work in united states</t>
+          <t>Are you able to obtain a Government Clearance</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1192,14 +1196,14 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>I am authorized to work in this country for any employer</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>high school/university/college degrees held</t>
+          <t>How many years of AWS experience do you have?</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1207,16 +1211,14 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Bachelor's in Computer Science</t>
-        </is>
+      <c r="C48" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>submit a drug screen and background check?</t>
+          <t>have a navy qual/cert ordnance certification?</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1226,48 +1228,48 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>what is your availability to begin working</t>
+          <t>eligible to be employed in the united states?</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Anytime- Immediately.</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>participate in any stage of a procurement</t>
+          <t>list the cloud providers you have experience</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>AWS, Azure, Digital Ocean</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>required citizenship status is US Citizen</t>
+          <t>How many years of Robotic Process Automation</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1275,33 +1277,31 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Yes- and I have a DHS Public Trust</t>
-        </is>
+      <c r="C52" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>do you have us. gov't security clearance?</t>
+          <t>level of clearance have you held previously?</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>what type of employment are you seeking?</t>
+          <t>currently hold an active security clearance?</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1311,31 +1311,31 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>full time</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>may we inquire of your present employer?</t>
+          <t>high school/university/college degrees held</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Bachelor's in Computer Science</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>current position for at least 12 months?</t>
+          <t>are you authorized to work in united states</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1345,14 +1345,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>I am authorized to work in this country for any employer</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>authorized to work in the United States</t>
+          <t>submit a drug screen and background check?</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1369,7 +1369,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>active and relevant certifications held</t>
+          <t>what is your availability to begin working</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1377,63 +1377,71 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Anytime- Immediately.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>what is your annual salary requirement?</t>
+          <t>special courses, seminars, and/or training</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>Selenium Automation with Python: I built a desktop automation tool using Selenium, Tkinter, and pandas to auto-fill web applications. This involved dynamic element detection, Chrome remote debugging, and advanced use of XPath, waits, and exception handling.
+Section 508 &amp; WCAG Accessibility Training: I received training while working on federal systems to implement accessibility standards including ARIA roles, keyboard navigation, and screen reader compatibility.
+Agile/Scrum Methodologies: I’ve worked in Agile environments using sprints, story points, and daily standups to deliver features incrementally and collaboratively.
+Cloud &amp; DevOps Tooling: I created automation tools using Python, AWS (boto3), and Docker during my internship, which improved infrastructure management and testing efficiency.
+Compiler Design (LEX/YACC): I completed a university project using LEX and YACC to build interpreters for custom programming and assembly languages, reinforcing my understanding of parsing and low-level architecture.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>when would you be able to start working</t>
+          <t>do you have us. gov't security clearance?</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>how did you hear about this position? *</t>
+          <t>required citizenship status is US Citizen</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>i have not entered into any non-compet</t>
+          <t>participate in any stage of a procurement</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1443,31 +1451,31 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>how many years of relevant experience</t>
+          <t>may we inquire of your present employer?</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>live in the united states of america?</t>
+          <t>what type of employment are you seeking?</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1477,31 +1485,31 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>full time</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>years of linux programming experience</t>
+          <t>current position for at least 12 months?</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>security clearance you currently hold</t>
+          <t>active and relevant certifications held</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1509,33 +1517,29 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>DHS Public Trust</t>
-        </is>
-      </c>
+      <c r="C66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Are you authorized to work in the US?</t>
+          <t>what is your annual salary requirement?</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>120</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>current level of an active clearance?</t>
+          <t>when would you be able to start working</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1545,14 +1549,14 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>What is your current location (State)</t>
+          <t>authorized to work in the United States</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1562,14 +1566,14 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>virginia</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>how did you hear about the position?</t>
+          <t>how did you hear about this position? *</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1579,14 +1583,14 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>other</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Do you have the necessary experience</t>
+          <t>knowledge of devops and ci/cd pipelines</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1603,7 +1607,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Will you be able to reliably commute</t>
+          <t>i have not entered into any non-compet</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1620,58 +1624,58 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Have you previously been employed by</t>
+          <t>level clearance do you currently hold?</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>other</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>please select your disability status</t>
+          <t>how many years of relevant experience</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>I don't have a disability</t>
+          <t>4-5</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>highest level of education obtained?</t>
+          <t>What is your current location (State)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Bachelor</t>
+          <t>virginia</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>when would you be available to begin</t>
+          <t>current level of an active clearance?</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -1681,14 +1685,14 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Total years of relative experience?</t>
+          <t>live in the united states of america?</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -1698,14 +1702,14 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2+</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Do you hold an active TS/SCI w/FSP?</t>
+          <t>security clearance you currently hold</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1715,14 +1719,14 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>no, I have a DHS Public Trust</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>is your clearance currently active?</t>
+          <t>experience in software re-engineering</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -1739,39 +1743,41 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>eligible to obtain a public trust?</t>
+          <t>years of linux programming experience</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>What are your salary expectations?</t>
+          <t>Are you authorized to work in the US?</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C81" t="n">
-        <v>120000</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Do you have a TS/SCI with CI poly?</t>
+          <t>Will you be able to reliably commute</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -1781,14 +1787,14 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Do you have a valid US Citizenship</t>
+          <t>Have you previously been employed by</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -1798,14 +1804,14 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>years of relevant work experience</t>
+          <t>when would you be available to begin</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -1815,14 +1821,14 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>former employee of any government</t>
+          <t>Do you have the necessary experience</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -1832,14 +1838,14 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>never</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>please select your veteran status</t>
+          <t>please select your disability status</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -1849,39 +1855,292 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>I am not a protected veteran</t>
+          <t>I don't have a disability</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>please provide an non voip number</t>
+          <t>highest level of education obtained?</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>703-473-5140</t>
+          <t>Bachelor</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
+          <t>how did you hear about the position?</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Do you hold an active TS/SCI w/FSP?</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>no, I have a DHS Public Trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Total years of relative experience?</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2+</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>is your clearance currently active?</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Do you have a TS/SCI with CI poly?</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Do you have a valid US Citizenship</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>What are your salary expectations?</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>eligible to obtain a public trust?</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>years of relevant work experience</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>please select your veteran status</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>I am not a protected veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>please provide an non voip number</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>703-473-5140</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>statement for maryland applicants</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Acknowledged by applicant</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>do you have an irs mbi clearance?</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>former employee of any government</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>never</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>do you have relatives employed by</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
           <t>please copy and paste your resume</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>textarea</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>Raqib Zaman
 Lorton, VA | 703-473-5140 | raqib.zaman@gmail.com LinkedIn: linkedin.com/in/raqibzaman 
@@ -1945,280 +2204,27 @@
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>do you have an irs mbi clearance?</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>how did you hear about this job?</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>online search</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>we may use sms during the hiring</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>have an active secret clearance?</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>position requires US citizenship</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Yes- and I have a DHS Public Trust</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>worked for this company before?</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>When are you available to start</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Anytime</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>Do you have a Bachelor's Degree</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>do you have federal experience?</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>years of ServiceNow experience</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C98" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>what is your desired salary? *</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Annual</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>receiving text communications</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>please enter the amount ($) *</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>120000</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Are you located in Arizona? *</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Are you a protected Veteran?</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>how did you hear about us? *</t>
+          <t>how did you hear about this job?</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>online search</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>are you a military veteran?</t>
+          <t>we may use sms during the hiring</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2228,31 +2234,31 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>are you currently employed?</t>
+          <t>position requires US citizenship</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>type of employment desired</t>
+          <t>have an active secret clearance?</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2262,14 +2268,14 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>full-time</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>require a visa sponsorship</t>
+          <t>worked for this company before?</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2286,7 +2292,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>certifications do you have</t>
+          <t>When are you available to start</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2296,19 +2302,19 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>Anytime</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>will you be able to start</t>
+          <t>do you have federal experience?</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2320,41 +2326,39 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>preferred contact method</t>
+          <t>Do you have a Bachelor's Degree</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Phone, anytime.</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Protected Veteran Status</t>
+          <t>years of ServiceNow experience</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>I am not a protected veteran</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>do you want to opt-in? *</t>
+          <t>what is your desired salary? *</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2364,14 +2368,14 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Annual</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>require visa sponsorship</t>
+          <t>location are you applying for?</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -2381,48 +2385,48 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Washington, DC</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>professional references</t>
+          <t>have you ever been employed by</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Bunmi Toye: (443)-929-3603, John Garber: john.d.garber@gmail.com 575-649-0811, Nicole Jacobs: (703)-801-3421, Sejal Dhawan: sejaldhawan98@gmail.com</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>review your application</t>
+          <t>please enter the amount ($) *</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>review your application</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>require any sponsorship</t>
+          <t>Are you located in Arizona? *</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -2439,7 +2443,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>best method to contact</t>
+          <t>held a clearance in the past?</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2449,14 +2453,14 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>able to work remotely</t>
+          <t>receiving text communications</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -2473,58 +2477,58 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>desired compensation?</t>
+          <t>are you currently employed by</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>120000</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>if you were referred</t>
+          <t>Are you a protected Veteran?</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>active DoD clearance</t>
+          <t>how did you hear about us? *</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Indeed</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>willing to relocate?</t>
+          <t>are you a military veteran?</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -2541,7 +2545,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>require sponsorship</t>
+          <t>are you currently employed?</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -2558,7 +2562,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>reside in the u.s.</t>
+          <t>require a visa sponsorship</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -2568,65 +2572,65 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>security clearance</t>
+          <t>certifications do you have</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Public Trust</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>level of education</t>
+          <t>highschool name &amp; location</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>4 Year University</t>
+          <t>Robert E. Lee (John R. Lewis) High School. 6540 Franconia Rd, Springfield, VA 22150</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>current clearance</t>
+          <t>type of employment desired</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>full-time</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>disability status</t>
+          <t>legally authorized to work</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -2636,31 +2640,31 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Disability Status</t>
+          <t>will you be able to start</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>No, I do not have a disability and have not had one in the past</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>18 years or older</t>
+          <t>do you want to opt-in? *</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -2677,7 +2681,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>able to relocate</t>
+          <t>require visa sponsorship</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -2687,48 +2691,48 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Doesn't apply</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ts/sci with poly</t>
+          <t>preferred contact method</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Phone, anytime.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>select your race</t>
+          <t>united states government</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Asian</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>driver's license</t>
+          <t>Protected Veteran Status</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -2738,44 +2742,48 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>I am not a protected veteran</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Clearance Level</t>
+          <t>review your application</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr"/>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>review your application</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>date available</t>
+          <t>require any sponsorship</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>highest degree</t>
+          <t>professional references</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -2785,31 +2793,31 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Bachelors Degree in Computer Science</t>
+          <t>Bunmi Toye: 443-929-3603, John Garber: john.d.garber@gmail.com 575-649-0811, Nicole Jacobs: 703-801-3421</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>veteran status</t>
+          <t>Supervisor Name &amp; Title</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>not a protected veteran</t>
+          <t>Bunmi Toye, Scrum Master</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>best method to contact</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -2819,65 +2827,65 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>I am not a veteran</t>
+          <t>email</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>veteran status</t>
+          <t>able to work remotely</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>not a veteran</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>u.s. citizen</t>
+          <t>desired compensation?</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>willing to relocate?</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>cover letter</t>
+          <t>active DoD clearance</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -2887,31 +2895,31 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>enter text</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>middle name</t>
+          <t>if you were referred</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>uz</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Desired Pay</t>
+          <t>how did you find out</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -2919,31 +2927,33 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C146" t="n">
-        <v>120000</v>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>US Citizen</t>
+          <t>Latest Employer Name</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>CVP (Customer Value Partners)</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>disability</t>
+          <t>require sponsorship</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -2960,15 +2970,604 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
+          <t>required to sponsor</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>related experience</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>security clearance</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Public Trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>reason for leaving</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>laid off, end of contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>reside in the u.s.</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>level of education</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>4 Year University</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Disability Status</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>No, I do not have a disability and have not had one in the past</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>disability status</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>18 years or older</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>did you graduate?</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>current clearance</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>DHS Public Trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>method of contact</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>ethnic background</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>able to relocate</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Doesn't apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>select your race</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>ts/sci with poly</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>current location</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Lorton, VA</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>driver's license</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>may we contact?</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Clearance Level</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>veteran status</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>not a veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>date available</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Veteran Status</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>I am not a veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>veteran status</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>not a protected veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>highest degree</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Bachelors Degree in Computer Science</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>united states</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>cover letter</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
           <t>enter text</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>u.s. citizen</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Apply anyway</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Apply anyway</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>I understand</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>I understand</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>shareholder</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>middle name</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>uz</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>proficiency</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Desired Pay</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>u.s citizen</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>enter text</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
         <is>
           <t>[cover letter]</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
+      <c r="C184" t="inlineStr">
         <is>
           <t>Dear Hiring Manager,
 I am writing to express my interest in the Software Developer position at [Company Name], as advertised. With over four years of hands-on experience developing full stack enterprise web applications for federal clients, I bring a strong foundation in ASP.NET MVC, C#, JavaScript, SQL, and accessibility standards. My technical proficiency and dedication to delivering high-quality, compliant software solutions align well with your team’s mission.
@@ -2981,216 +3580,403 @@
         </is>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>experience</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>average</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>disability</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>US Citizen</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
         <is>
           <t>Bachelors Degree</t>
         </is>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>job title</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
         <is>
           <t>ethnicity</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B191" t="inlineStr">
         <is>
           <t>select-one</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C191" t="inlineStr">
         <is>
           <t>asian</t>
         </is>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
+    <row r="192">
+      <c r="A192" t="inlineStr">
         <is>
           <t>Continue</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
+      <c r="B192" t="inlineStr">
         <is>
           <t>button</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
+      <c r="C192" t="inlineStr">
         <is>
           <t>Continue</t>
         </is>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>new jobs</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>18 years</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>consent</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>i consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>I agree</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>I understand</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
         <is>
           <t>Gender</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>suffix</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
         <is>
           <t>felony</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>suffix</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr"/>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
+    <row r="201">
+      <c r="A201" t="inlineStr">
         <is>
           <t>salary</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C156" t="n">
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
         <v>120000</v>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
         <is>
           <t>Race</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B203" t="inlineStr">
         <is>
           <t>select-one</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
+      <c r="C203" t="inlineStr">
         <is>
           <t>Asian</t>
         </is>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
+    <row r="204">
+      <c r="A204" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr">
+      <c r="B204" t="inlineStr">
         <is>
           <t>select-one</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
+      <c r="C204" t="inlineStr">
         <is>
           <t>Anytime (8am - 9pm)</t>
         </is>
       </c>
     </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
+    <row r="205">
+      <c r="A205" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
         <is>
           <t>Raqib Zaman</t>
         </is>
       </c>
     </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
+    <row r="206">
+      <c r="A206" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
         <is>
           <t>[current date]</t>
         </is>
       </c>
     </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
+    <row r="207">
+      <c r="A207" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr">
+      <c r="B207" t="inlineStr">
         <is>
           <t>select-one</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
+      <c r="C207" t="inlineStr">
         <is>
           <t>Weekday</t>
         </is>
       </c>
     </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
+    <row r="208">
+      <c r="A208" t="inlineStr">
         <is>
           <t>zip</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
         <is>
           <t>22079</t>
         </is>

</xml_diff>

<commit_message>
Added checkbox input handling
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C208"/>
+  <dimension ref="A1:C221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -699,56 +699,58 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>How many years of modern JavaScript experience do you have?</t>
+          <t>describe what you'd like to be doing on a day-to-day basis *</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>6</v>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>On a day-to-day basis, I want to work on full stack development projects, building and improving web applications using ASP.NET MVC, C#, JavaScript, and SQL. I enjoy creating clean, efficient code for both front-end interfaces and back-end services that solve real user problems and enhance functionality.
+I like collaborating closely with team members through agile processes like daily stand-ups and code reviews, ensuring that features meet business requirements and maintain high quality. Troubleshooting, debugging, and optimizing code and database queries are important parts of my routine to keep applications running smoothly.
+Additionally, I want to contribute to automation and deployment efforts using tools like Docker and AWS, while continuously learning new technologies and best practices to improve my skills and deliver scalable, maintainable solutions.</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>are you able to perform the essential functions of the job</t>
+          <t>how many years of experience do you have in a saas company?</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>do you have an active ts/sci clearance and fs polygraph? *</t>
+          <t>How many years of modern JavaScript experience do you have?</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>experience with code vulnerability mitigation/remediation</t>
+          <t>are you able to perform the essential functions of the job</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -765,22 +767,24 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>How many years of Microservices experience do you have?</t>
+          <t>do you have an active ts/sci clearance and fs polygraph? *</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>are you able to commute daily to the location indicated</t>
+          <t>experience with code vulnerability mitigation/remediation</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -797,7 +801,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>if presently employed, why are you considering leaving?</t>
+          <t>How many years of Microservices experience do you have?</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -805,16 +809,14 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>not applicable</t>
-        </is>
+      <c r="C23" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>require any immigration related support or sponsorship</t>
+          <t>are you able to commute daily to the location indicated</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -824,24 +826,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Do you have 1 or more of the following certifications?</t>
+          <t>if presently employed, why are you considering leaving?</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
@@ -878,7 +880,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Do you currently have a relative or spouse working at</t>
+          <t>require any immigration related support or sponsorship</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -895,72 +897,74 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>How many years of applicable experience do you have?</t>
+          <t>Do you have 1 or more of the following certifications?</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Do you currently have a relative or spouse working at</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>How many years of applicable experience do you have?</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>do you want to tell us anything else about yourself?</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>textarea</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Automated Job Application Tool – Personal Project | May 2025 – Present
 Developed a Python desktop automation tool using Selenium, Tkinter, and pandas to auto-fill online job applications. Designed a GUI to control flow and dynamically update form data from Excel files. Implemented DOM scraping and fuzzy string matching to identify and interact with visible form elements (textboxes, radio buttons, dropdowns). Enabled Chrome remote debugging for resilient, real-time automation and built intelligent logic to skip irrelevant pages and adapt behavior based on the page URL. Link: github.com/RaqibZaman/AutomateJobApplication</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Do you have an active Top Secret security clearance?</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>applied DevOps professional experience do you have?</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>4</v>
-      </c>
-    </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>by submitting your application you hereby certify</t>
+          <t>Do you have an active Top Secret security clearance?</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -970,14 +974,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>accept</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>How many years of MongoDB experience do you have?</t>
+          <t>applied DevOps professional experience do you have?</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -986,45 +990,47 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>How many years of airflow experience do you have?</t>
+          <t>top 3 things you look for when selecting a new job</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>0</v>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>I look for roles where I can work on technically challenging projects that serve a meaningful purpose, particularly in the public sector or high-availability enterprise systems. I enjoy contributing to full stack solutions using technologies like ASP.NET MVC, C#, JavaScript, and SQL, especially when the work involves features like data reporting, system automation, or accessibility compliance (Section 508/WCAG). I am most fulfilled when my code directly improves usability, efficiency, or compliance for end users.
+Additionally, I value teams that emphasize clean architecture, code reviews, and agile methodologies like Scrum. I appreciate environments that apply DevOps practices such as CI/CD pipelines, Docker, and cloud deployments with AWS or Azure. Teams that use tools like Git, JIRA, and automated testing to improve velocity and maintainability are where I do my best work. A culture that promotes documentation, peer collaboration, and accountability helps me grow while enabling high-quality, sustainable development.
+Finally, I seek positions that encourage both vertical and horizontal growth. This includes expanding into newer frameworks like React or Blazor, improving my cloud infrastructure skills, or exploring adjacent areas such as cybersecurity or performance tuning. I am particularly drawn to roles that offer exposure to different layers of the stack or to evolving federal standards. This allows me to continuously deepen and broaden my expertise.</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>lived in the us for at least the last three years</t>
+          <t>How many years of MongoDB experience do you have?</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Do you have 5+ years of Microsoft Power Platform</t>
+          <t>by submitting your application you hereby certify</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1034,31 +1040,29 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>accept</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>linux scripting language are you most proficient</t>
+          <t>How many years of airflow experience do you have?</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>textarea</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Bash, Python, and looking into Lua</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Do you have 8+ years of Microsoft Power Platform</t>
+          <t>lived in the us for at least the last three years</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1068,76 +1072,80 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>How many years of Python experience do you have?</t>
+          <t>linux scripting language are you most proficient</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>4</v>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Bash, Python, and looking into Lua</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Please list any relevant certifications you hold</t>
+          <t>Do you have 5+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>do you reside in one of the following us states</t>
+          <t>How many years of Python experience do you have?</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>please provide us with a copy of your agreement</t>
+          <t>Do you have 8+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>button</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Confirm Home Address (Street, City, State, Zip)</t>
+          <t>Please list any relevant certifications you hold</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1147,89 +1155,87 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>8324 Middle Ruddings Dr, Lorton, VA, 22079</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>How many years of Java experience do you have?</t>
+          <t>do you reside in one of the following us states</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>5</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Are you eligible to work in the United States?</t>
+          <t>please provide us with a copy of your agreement</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Are you able to obtain a Government Clearance</t>
+          <t>Confirm Home Address (Street, City, State, Zip)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>8324 Middle Ruddings Dr, Lorton, VA, 22079</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>How many years of AWS experience do you have?</t>
+          <t>Are you eligible to work in the United States?</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>have a navy qual/cert ordnance certification?</t>
+          <t>How many years of Java experience do you have?</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -1252,24 +1258,24 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>list the cloud providers you have experience</t>
+          <t>have a navy qual/cert ordnance certification?</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>AWS, Azure, Digital Ocean</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>How many years of Robotic Process Automation</t>
+          <t>How many years of AWS experience do you have?</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1278,23 +1284,23 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>level of clearance have you held previously?</t>
+          <t>Are you able to obtain a Government Clearance</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1318,83 +1324,132 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>high school/university/college degrees held</t>
+          <t>level of clearance have you held previously?</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Bachelor's in Computer Science</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>are you authorized to work in united states</t>
+          <t>How many years of Robotic Process Automation</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>I am authorized to work in this country for any employer</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>submit a drug screen and background check?</t>
+          <t>list the cloud providers you have experience</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>AWS, Azure, Digital Ocean</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>what is your availability to begin working</t>
+          <t>are you authorized to work in united states</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Anytime- Immediately.</t>
+          <t>I am authorized to work in this country for any employer</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>high school/university/college degrees held</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Bachelor's in Computer Science</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>what is your availability to begin working</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Anytime- Immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>submit a drug screen and background check?</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>special courses, seminars, and/or training</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>textarea</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>Selenium Automation with Python: I built a desktop automation tool using Selenium, Tkinter, and pandas to auto-fill web applications. This involved dynamic element detection, Chrome remote debugging, and advanced use of XPath, waits, and exception handling.
 Section 508 &amp; WCAG Accessibility Training: I received training while working on federal systems to implement accessibility standards including ARIA roles, keyboard navigation, and screen reader compatibility.
@@ -1404,61 +1459,10 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>do you have us. gov't security clearance?</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>required citizenship status is US Citizen</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Yes- and I have a DHS Public Trust</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>participate in any stage of a procurement</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>may we inquire of your present employer?</t>
+          <t>participate in any stage of a procurement</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1468,14 +1472,14 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>what type of employment are you seeking?</t>
+          <t>do you have us. gov't security clearance?</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1485,90 +1489,90 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>full time</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>current position for at least 12 months?</t>
+          <t>required citizenship status is US Citizen</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>active and relevant certifications held</t>
+          <t>what type of employment are you seeking?</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>full time</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>what is your annual salary requirement?</t>
+          <t>current position for at least 12 months?</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>when would you be able to start working</t>
+          <t>may we inquire of your present employer?</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>authorized to work in the United States</t>
+          <t>active and relevant certifications held</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1590,75 +1594,75 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>knowledge of devops and ci/cd pipelines</t>
+          <t>what is your annual salary requirement?</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>120</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>i have not entered into any non-compet</t>
+          <t>when would you be able to start working</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>level clearance do you currently hold?</t>
+          <t>authorized to work in the United States</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>how many years of relevant experience</t>
+          <t>knowledge of devops and ci/cd pipelines</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>What is your current location (State)</t>
+          <t>require any type of work authorization</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1668,41 +1672,41 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>virginia</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>current level of an active clearance?</t>
+          <t>i have not entered into any non-compet</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>live in the united states of america?</t>
+          <t>level clearance do you currently hold?</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>other</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1730,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>experience in software re-engineering</t>
+          <t>live in the united states of america?</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -1760,7 +1764,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Are you authorized to work in the US?</t>
+          <t>What is your current location (State)</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -1770,65 +1774,65 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>virginia</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Will you be able to reliably commute</t>
+          <t>how many years of relevant experience</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>4-5</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Have you previously been employed by</t>
+          <t>current level of an active clearance?</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>when would you be available to begin</t>
+          <t>not interested in doing for this role</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>No, I am quite interested in all new technologies, especially machine learning and AI</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Do you have the necessary experience</t>
+          <t>experience in software re-engineering</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -1845,7 +1849,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>please select your disability status</t>
+          <t>Are you authorized to work in the US?</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -1855,31 +1859,31 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>I don't have a disability</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>highest level of education obtained?</t>
+          <t>Have you previously been employed by</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Bachelor</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>how did you hear about the position?</t>
+          <t>Do you have the necessary experience</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -1889,48 +1893,48 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Do you hold an active TS/SCI w/FSP?</t>
+          <t>Will you be able to reliably commute</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>no, I have a DHS Public Trust</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Total years of relative experience?</t>
+          <t>when would you be available to begin</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2+</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>is your clearance currently active?</t>
+          <t>how did you hear about the position?</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -1940,14 +1944,14 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>indeed</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Do you have a TS/SCI with CI poly?</t>
+          <t>please select your disability status</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -1957,46 +1961,48 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>I don't have a disability</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Do you have a valid US Citizenship</t>
+          <t>highest level of education obtained?</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Bachelor</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>What are your salary expectations?</t>
+          <t>Total years of relative experience?</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C94" t="n">
-        <v>120000</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2+</t>
+        </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>eligible to obtain a public trust?</t>
+          <t>is your clearance currently active?</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2013,7 +2019,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>years of relevant work experience</t>
+          <t>Do you hold an active TS/SCI w/FSP?</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2023,14 +2029,14 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>no, I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>please select your veteran status</t>
+          <t>Do you have a TS/SCI with CI poly?</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2040,31 +2046,29 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>I am not a protected veteran</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>please provide an non voip number</t>
+          <t>What are your salary expectations?</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>textarea</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>703-473-5140</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>statement for maryland applicants</t>
+          <t>Do you have a valid US Citizenship</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2074,14 +2078,14 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Acknowledged by applicant</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>do you have an irs mbi clearance?</t>
+          <t>eligible to obtain a public trust?</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2091,24 +2095,24 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>former employee of any government</t>
+          <t>years of relevant work experience</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>never</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -2132,15 +2136,83 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t>please select your veteran status</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>I am not a protected veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>please provide an non voip number</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>703-473-5140</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>statement for maryland applicants</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Acknowledged by applicant</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>former employee of any government</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>never</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
           <t>please copy and paste your resume</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B107" t="inlineStr">
         <is>
           <t>textarea</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>Raqib Zaman
 Lorton, VA | 703-473-5140 | raqib.zaman@gmail.com LinkedIn: linkedin.com/in/raqibzaman 
@@ -2204,78 +2276,10 @@
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>how did you hear about this job?</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>online search</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>we may use sms during the hiring</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>position requires US citizenship</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>Yes- and I have a DHS Public Trust</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>have an active secret clearance?</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>worked for this company before?</t>
+          <t>do you have an irs mbi clearance?</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2292,7 +2296,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>When are you available to start</t>
+          <t>how did you hear about this job?</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2302,31 +2306,31 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Anytime</t>
+          <t>online search</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>do you have federal experience?</t>
+          <t>position requires US citizenship</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Do you have a Bachelor's Degree</t>
+          <t>we may use sms during the hiring</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2343,22 +2347,24 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>years of ServiceNow experience</t>
+          <t>have an active secret clearance?</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C112" t="n">
-        <v>1</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>what is your desired salary? *</t>
+          <t>worked for this company before?</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2368,14 +2374,14 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>location are you applying for?</t>
+          <t>do you have federal experience?</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -2385,65 +2391,63 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>have you ever been employed by</t>
+          <t>When are you available to start</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Anytime</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>please enter the amount ($) *</t>
+          <t>Do you have a Bachelor's Degree</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>120000</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Are you located in Arizona? *</t>
+          <t>years of ServiceNow experience</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>held a clearance in the past?</t>
+          <t>location are you applying for?</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2453,14 +2457,14 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Washington, DC</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>receiving text communications</t>
+          <t>what is your desired salary? *</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -2470,14 +2474,14 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Annual</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>are you currently employed by</t>
+          <t>have you ever been employed by</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -2494,41 +2498,41 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Are you a protected Veteran?</t>
+          <t>please enter the amount ($) *</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>how did you hear about us? *</t>
+          <t>held a clearance in the past?</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>are you a military veteran?</t>
+          <t>are you currently employed by</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -2545,7 +2549,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>are you currently employed?</t>
+          <t>do you live in ca, hi, or ak?</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -2562,7 +2566,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>require a visa sponsorship</t>
+          <t>Are you located in Arizona? *</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -2579,41 +2583,41 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>certifications do you have</t>
+          <t>receiving text communications</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>highschool name &amp; location</t>
+          <t>how did you hear about us? *</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Robert E. Lee (John R. Lewis) High School. 6540 Franconia Rd, Springfield, VA 22150</t>
+          <t>Indeed</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>type of employment desired</t>
+          <t>Are you a protected Veteran?</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -2623,14 +2627,14 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>full-time</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>legally authorized to work</t>
+          <t>are you currently employed?</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -2640,48 +2644,48 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>will you be able to start</t>
+          <t>are you a military veteran?</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>do you want to opt-in? *</t>
+          <t>certifications do you have</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>require visa sponsorship</t>
+          <t>type of employment desired</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -2691,14 +2695,14 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>full-time</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>preferred contact method</t>
+          <t>highschool name &amp; location</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -2708,14 +2712,14 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Phone, anytime.</t>
+          <t>Robert E. Lee (John R. Lewis) High School. 6540 Franconia Rd, Springfield, VA 22150</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>united states government</t>
+          <t>legally authorized to work</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -2725,14 +2729,14 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Protected Veteran Status</t>
+          <t>require a visa sponsorship</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -2742,31 +2746,31 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>I am not a protected veteran</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>review your application</t>
+          <t>will you be able to start</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>review your application</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>require any sponsorship</t>
+          <t>require visa sponsorship</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -2783,7 +2787,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>professional references</t>
+          <t>preferred contact method</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -2793,31 +2797,31 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Bunmi Toye: 443-929-3603, John Garber: john.d.garber@gmail.com 575-649-0811, Nicole Jacobs: 703-801-3421</t>
+          <t>Phone, anytime.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Supervisor Name &amp; Title</t>
+          <t>united states government</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Bunmi Toye, Scrum Master</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>best method to contact</t>
+          <t>do you want to opt-in? *</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -2827,14 +2831,14 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>able to work remotely</t>
+          <t>Protected Veteran Status</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -2844,31 +2848,31 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>I am not a protected veteran</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>desired compensation?</t>
+          <t>what state do you reside</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>checkbox</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>120000</t>
+          <t>Virginia</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>willing to relocate?</t>
+          <t>require any sponsorship</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -2885,7 +2889,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>active DoD clearance</t>
+          <t>eligible for employment</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -2895,31 +2899,31 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>if you were referred</t>
+          <t>Supervisor Name &amp; Title</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>Bunmi Toye, Scrum Master</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>how did you find out</t>
+          <t>professional references</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -2929,48 +2933,48 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>Bunmi Toye: 443-929-3603, John Garber: john.d.garber@gmail.com 575-649-0811, Nicole Jacobs: 703-801-3421</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Latest Employer Name</t>
+          <t>review your application</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>button</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>CVP (Customer Value Partners)</t>
+          <t>review your application</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>require sponsorship</t>
+          <t>why are you interested</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>I'm interested in working with your team because it aligns with my experience building scalable, accessible web applications using ASP.NET MVC, C#, JavaScript, and SQL—especially in federal environments like DHS EPHP DSS and FPS PTS. I enjoy solving real-world problems through full stack development, such as implementing dynamic form logic, exportable reports, and Section 508 compliance. I’m excited by opportunities to contribute to meaningful software that improves user workflows, meets client standards, and supports long-term maintainability.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>required to sponsor</t>
+          <t>best method to contact</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -2980,48 +2984,48 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>email</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>related experience</t>
+          <t>Location (city, state)</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Lorton, VA</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>security clearance</t>
+          <t>able to work remotely</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Public Trust</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>reason for leaving</t>
+          <t>desired compensation?</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -3031,48 +3035,48 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>laid off, end of contract</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>reside in the u.s.</t>
+          <t>if you were referred</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>level of education</t>
+          <t>how did you find out</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>4 Year University</t>
+          <t>indeed</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Disability Status</t>
+          <t>active DoD clearance</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -3082,31 +3086,31 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>No, I do not have a disability and have not had one in the past</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>disability status</t>
+          <t>Latest Employer Name</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>CVP (Customer Value Partners)</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>18 years or older</t>
+          <t>willing to relocate?</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -3116,14 +3120,14 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>did you graduate?</t>
+          <t>required to sponsor</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -3133,65 +3137,65 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>current clearance</t>
+          <t>require sponsorship</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>method of contact</t>
+          <t>level of education</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>4 Year University</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ethnic background</t>
+          <t>reason for leaving</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>asian</t>
+          <t>laid off, end of contract</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>able to relocate</t>
+          <t>reside in the u.s.</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -3201,14 +3205,14 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Doesn't apply</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>select your race</t>
+          <t>security clearance</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -3218,14 +3222,14 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Asian</t>
+          <t>Public Trust</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ts/sci with poly</t>
+          <t>related experience</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -3235,31 +3239,31 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>current location</t>
+          <t>method of contact</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Lorton, VA</t>
+          <t>Email</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>driver's license</t>
+          <t>did you graduate?</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -3276,71 +3280,75 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>may we contact?</t>
+          <t>current clearance</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Clearance Level</t>
+          <t>ethnic background</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr"/>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>asian</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>veteran status</t>
+          <t>18 years or older</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>not a veteran</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>date available</t>
+          <t>disability status</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>Disability Status</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -3350,14 +3358,14 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>I am not a veteran</t>
+          <t>No, I do not have a disability and have not had one in the past</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>veteran status</t>
+          <t>driver's license</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -3367,31 +3375,31 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>not a protected veteran</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>highest degree</t>
+          <t>ts/sci with poly</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Bachelors Degree in Computer Science</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>united states</t>
+          <t>able to relocate</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -3401,65 +3409,65 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Doesn't apply</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>cover letter</t>
+          <t>select your race</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>enter text</t>
+          <t>Asian</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>u.s. citizen</t>
+          <t>current location</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Lorton, VA</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>may we contact?</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>I understand</t>
+          <t>Clearance Level</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -3467,33 +3475,29 @@
           <t>radio</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>I understand</t>
-        </is>
-      </c>
+      <c r="C178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>shareholder</t>
+          <t>highest degree</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Bachelors Degree in Computer Science</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>middle name</t>
+          <t>date available</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -3503,14 +3507,14 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>uz</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>proficiency</t>
+          <t>Veteran Status</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -3520,54 +3524,275 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>I am not a veteran</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Desired Pay</t>
+          <t>elevator pitch</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C182" t="n">
-        <v>120000</v>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>I’m Raqib Zaman, a detail-oriented full stack software developer with over four years of experience building enterprise web applications, primarily using ASP.NET MVC, C#, JavaScript, and SQL. I specialize in creating accessible, high-quality solutions for federal clients, ensuring compliance with standards like Section 508 while delivering features that improve efficiency and user experience. Beyond development, I have hands-on experience with DevOps tools like Docker and AWS, and have developed automation tools using Python and Selenium to streamline repetitive tasks and improve workflow efficiency. I’m passionate about writing clean, maintainable code that solves real-world problems and drives positive impact.</t>
+        </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>u.s citizen</t>
+          <t>veteran status</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>not a veteran</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
+          <t>veteran status</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>not a protected veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>how you found</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>indeed.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>united states</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>u.s. citizen</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Apply anyway</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Apply anyway</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>cover letter</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
           <t>enter text</t>
         </is>
       </c>
-      <c r="B184" t="inlineStr">
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>I understand</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>I understand</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>middle name</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>uz</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>u.s citizen</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>shareholder</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Desired Pay</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>proficiency</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>US Citizen</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>enter text</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
         <is>
           <t>[cover letter]</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr">
+      <c r="C197" t="inlineStr">
         <is>
           <t>Dear Hiring Manager,
 I am writing to express my interest in the Software Developer position at [Company Name], as advertised. With over four years of hands-on experience developing full stack enterprise web applications for federal clients, I bring a strong foundation in ASP.NET MVC, C#, JavaScript, SQL, and accessibility standards. My technical proficiency and dedication to delivering high-quality, compliant software solutions align well with your team’s mission.
@@ -3580,231 +3805,10 @@
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>experience</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>average</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>disability</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>US Citizen</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>Bachelors Degree</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>job title</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>Full Stack Developer</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>ethnicity</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>asian</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>Continue</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>button</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>Continue</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>new jobs</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>18 years</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>consent</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>i consent</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>I agree</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>I understand</t>
-        </is>
-      </c>
-    </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>disability</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -3814,144 +3818,150 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>suffix</t>
+          <t>experience</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C199" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>average</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>felony</t>
+          <t>ethnicity</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>asian</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>salary</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C201" t="n">
-        <v>120000</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Bachelors Degree</t>
+        </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>agree</t>
+          <t>job title</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Race</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Asian</t>
+          <t>Bachelor</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>new jobs</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Anytime (8am - 9pm)</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>Continue</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>button</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Raqib Zaman</t>
+          <t>Continue</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>18 years</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>country</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -3961,22 +3971,237 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Weekday</t>
+          <t>United States</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
+          <t>I agree</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>I understand</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>consent</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>i consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>felony</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>suffix</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Anytime (8am - 9pm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Raqib Zaman</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Weekday</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
           <t>zip</t>
         </is>
       </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
         <is>
           <t>22079</t>
         </is>

</xml_diff>

<commit_message>
Need to try a different implementation that is more specific to the edge case with select WebElments
</commit_message>
<xml_diff>
--- a/Q_T_V.xlsx
+++ b/Q_T_V.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C246"/>
+  <dimension ref="A1:C261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,34 +499,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Do you have an active government clearance? Please list specifics in the text field</t>
+          <t>do you have experience designing, implementing, and maintaining aws-based solutions</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yes, DHS Public Trust</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>do you have experience designing, implementing, and maintaining aws-based solutions</t>
+          <t>Do you have an active government clearance? Please list specifics in the text field</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Yes, DHS Public Trust</t>
         </is>
       </c>
     </row>
@@ -1030,39 +1030,39 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>by submitting your application you hereby certify</t>
+          <t>How many years of airflow experience do you have?</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>accept</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>How many years of airflow experience do you have?</t>
+          <t>lived in the us for at least the last three years</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>lived in the us for at least the last three years</t>
+          <t>by submitting your application you hereby certify</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>accept</t>
         </is>
       </c>
     </row>
@@ -1096,83 +1096,83 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Do you have 5+ years of Microsoft Power Platform</t>
+          <t>Please list any relevant certifications you hold</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>How many years of Python experience do you have?</t>
+          <t>Do you have 5+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>4</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Do you have 8+ years of Microsoft Power Platform</t>
+          <t>How many years of Python experience do you have?</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Please list any relevant certifications you hold</t>
+          <t>Do you have 8+ years of Microsoft Power Platform</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>do you reside in one of the following us states</t>
+          <t>Confirm Home Address (Street, City, State, Zip)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>8324 Middle Ruddings Dr, Lorton, VA, 22079</t>
         </is>
       </c>
     </row>
@@ -1192,17 +1192,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Confirm Home Address (Street, City, State, Zip)</t>
+          <t>do you reside in one of the following us states</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>8324 Middle Ruddings Dr, Lorton, VA, 22079</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1407,34 +1407,34 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>what is your availability to begin working</t>
+          <t>submit a drug screen and background check?</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Anytime- Immediately.</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>submit a drug screen and background check?</t>
+          <t>what is your availability to begin working</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Anytime- Immediately.</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1462,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>participate in any stage of a procurement</t>
+          <t>do you have us. gov't security clearance?</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1472,48 +1472,48 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>do you have us. gov't security clearance?</t>
+          <t>required citizenship status is US Citizen</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Yes- and I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>required citizenship status is US Citizen</t>
+          <t>participate in any stage of a procurement</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Yes- and I have a DHS Public Trust</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>what type of employment are you seeking?</t>
+          <t>may we inquire of your present employer?</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1523,14 +1523,14 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>full time</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>current position for at least 12 months?</t>
+          <t>what type of employment are you seeking?</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1540,14 +1540,14 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>full time</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>may we inquire of your present employer?</t>
+          <t>current position for at least 12 months?</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1564,7 +1564,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>active and relevant certifications held</t>
+          <t>when would you be able to start working</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1572,12 +1572,16 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>how did you hear about this position? *</t>
+          <t>knowledge of devops and ci/cd pipelines</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1587,41 +1591,37 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>what is your annual salary requirement?</t>
+          <t>active and relevant certifications held</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>when would you be able to start working</t>
+          <t>what is your annual salary requirement?</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>120</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1645,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>knowledge of devops and ci/cd pipelines</t>
+          <t>how did you hear about this position? *</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1655,14 +1655,14 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>other</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>require any type of work authorization</t>
+          <t>i have not entered into any non-compet</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1672,58 +1672,58 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>i have not entered into any non-compet</t>
+          <t>level clearance do you currently hold?</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>other</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>level clearance do you currently hold?</t>
+          <t>require any type of work authorization</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>security clearance you currently hold</t>
+          <t>not interested in doing for this role</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>No, I am quite interested in all new technologies, especially machine learning and AI</t>
         </is>
       </c>
     </row>
@@ -1747,136 +1747,136 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>years of linux programming experience</t>
+          <t>What is your current location (State)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>virginia</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>What is your current location (State)</t>
+          <t>security clearance you currently hold</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>virginia</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>how many years of relevant experience</t>
+          <t>Are you authorized to work in the US?</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>current level of an active clearance?</t>
+          <t>experience in software re-engineering</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>not interested in doing for this role</t>
+          <t>years of linux programming experience</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>No, I am quite interested in all new technologies, especially machine learning and AI</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>experience in software re-engineering</t>
+          <t>how many years of relevant experience</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>4-5</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Are you authorized to work in the US?</t>
+          <t>current level of an active clearance?</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Have you previously been employed by</t>
+          <t>highest level of education obtained?</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Bachelor</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Will you be able to reliably commute</t>
+          <t>Have you previously been employed by</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>how did you hear about the position?</t>
+          <t>Will you be able to reliably commute</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -1944,14 +1944,14 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>please select your disability status</t>
+          <t>how did you hear about the position?</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -1961,48 +1961,48 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>I don't have a disability</t>
+          <t>indeed</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>highest level of education obtained?</t>
+          <t>please select your disability status</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Bachelor</t>
+          <t>I don't have a disability</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Total years of relative experience?</t>
+          <t>Do you hold an active TS/SCI w/FSP?</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2+</t>
+          <t>no, I have a DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>is your clearance currently active?</t>
+          <t>Total years of relative experience?</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2012,31 +2012,31 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>2+</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Do you hold an active TS/SCI w/FSP?</t>
+          <t>is your clearance currently active?</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>no, I have a DHS Public Trust</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Do you have a TS/SCI with CI poly?</t>
+          <t>eligible to obtain a public trust?</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>eligible to obtain a public trust?</t>
+          <t>Do you have a TS/SCI with CI poly?</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2398,34 +2398,34 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>When are you available to start</t>
+          <t>Do you have a Bachelor's Degree</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Anytime</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Do you have a Bachelor's Degree</t>
+          <t>When are you available to start</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Anytime</t>
         </is>
       </c>
     </row>
@@ -2449,33 +2449,33 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>years of ServiceNow experience</t>
+          <t>location are you applying for?</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C118" t="n">
-        <v>1</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Washington, DC</t>
+        </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>what is your desired salary? *</t>
+          <t>years of ServiceNow experience</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Annual</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="120">
@@ -2498,7 +2498,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>location are you applying for?</t>
+          <t>what is your desired salary? *</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -2508,48 +2508,48 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>Annual</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>please enter the amount ($) *</t>
+          <t>do you live in ca, hi, or ak?</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>120000</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>are you currently employed by</t>
+          <t>please enter the amount ($) *</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>do you live in ca, hi, or ak?</t>
+          <t>receiving text communications</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -2559,14 +2559,14 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Are you located in Arizona? *</t>
+          <t>are you currently employed by</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -2583,7 +2583,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>receiving text communications</t>
+          <t>held a clearance in the past?</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -2593,14 +2593,14 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>held a clearance in the past?</t>
+          <t>Are you located in Arizona? *</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -2617,54 +2617,54 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>how did you hear about us? *</t>
+          <t>where did you hear about us?</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Are you a protected Veteran?</t>
+          <t>how did you hear about us? *</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Indeed</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>where did you hear about us?</t>
+          <t>Are you a protected Veteran?</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>are you a military veteran?</t>
+          <t>are you currently employed?</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -2681,7 +2681,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>are you currently employed?</t>
+          <t>are you a military veteran?</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -2783,7 +2783,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>will you be able to start</t>
+          <t>message to the hiring team</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -2793,48 +2793,48 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Thank you for reviewing my application. I specialize in building scalable, accessible web applications using ASP.NET MVC, C#, and SQL. My approach involves distilling complex requirements into clean, maintainable code that aligns with both business logic and user experience. I’m also deeply interested in learning about AI and its implementation through Python TensorFlow, exploring ways to integrate LLMs into practical, automation-driven solutions. I’m excited to contribute both proven skills and forward-thinking ideas to your team.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>united states government</t>
+          <t>will you be able to start</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>require visa sponsorship</t>
+          <t>years of Agile experience</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Protected Veteran Status</t>
+          <t>united states government</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>I am not a protected veteran</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2902,24 +2902,24 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>years of test automation</t>
+          <t>Protected Veteran Status</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>I am not a protected veteran</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Supervisor Name &amp; Title</t>
+          <t>years of test automation</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -2929,14 +2929,14 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Bunmi Toye, Scrum Master</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>require any sponsorship</t>
+          <t>require visa sponsorship</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -2953,34 +2953,34 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>review your application</t>
+          <t>Supervisor Name &amp; Title</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>review your application</t>
+          <t>Bunmi Toye, Scrum Master</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>professional references</t>
+          <t>require any sponsorship</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Bunmi Toye: 443-929-3603, John Garber: john.d.garber@gmail.com 575-649-0811, Nicole Jacobs: 703-801-3421</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -3021,51 +3021,51 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>why are you interested</t>
+          <t>professional references</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>I'm interested in working with your team because it aligns with my experience building scalable, accessible web applications using ASP.NET MVC, C#, JavaScript, and SQL—especially in federal environments like DHS EPHP DSS and FPS PTS. I enjoy solving real-world problems through full stack development, such as implementing dynamic form logic, exportable reports, and Section 508 compliance. I’m excited by opportunities to contribute to meaningful software that improves user workflows, meets client standards, and supports long-term maintainability.</t>
+          <t>Bunmi Toye: 443-929-3603, John Garber: john.d.garber@gmail.com 575-649-0811, Nicole Jacobs: 703-801-3421</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Location (city, state)</t>
+          <t>review your application</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>button</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Lorton, VA</t>
+          <t>review your application</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>best method to contact</t>
+          <t>why are you interested</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>I'm interested in working with your team because it aligns with my experience building scalable, accessible web applications using ASP.NET MVC, C#, JavaScript, and SQL—especially in federal environments like DHS EPHP DSS and FPS PTS. I enjoy solving real-world problems through full stack development, such as implementing dynamic form logic, exportable reports, and Section 508 compliance. I’m excited by opportunities to contribute to meaningful software that improves user workflows, meets client standards, and supports long-term maintainability.</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>able to work remotely</t>
+          <t>best method to contact</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -3099,14 +3099,14 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>email</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>desired compensation?</t>
+          <t>years of C# experience</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -3116,27 +3116,31 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>120000</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>i decline to identify</t>
+          <t>Location (city, state)</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>checkbox</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Lorton, VA</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>willing to relocate?</t>
+          <t>able to work remotely</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -3146,31 +3150,27 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>how did you find out</t>
+          <t>i decline to identify</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
+          <t>checkbox</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Latest Employer Name</t>
+          <t>desired compensation?</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -3180,48 +3180,48 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>CVP (Customer Value Partners)</t>
+          <t>120000</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>control act of 1986?</t>
+          <t>how did you find out</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>indeed</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>if you were referred</t>
+          <t>willing to relocate?</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>active DoD clearance</t>
+          <t>control act of 1986?</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -3231,48 +3231,48 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>required to sponsor</t>
+          <t>Latest Employer Name</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>CVP (Customer Value Partners)</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>holder of clearance</t>
+          <t>if you were referred</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>DHS</t>
+          <t>not applicable</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>require sponsorship</t>
+          <t>active DoD clearance</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -3289,41 +3289,41 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>related experience</t>
+          <t>holder of clearance</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>DHS</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>level of education</t>
+          <t>required to sponsor</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>4 Year University</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>security clearance</t>
+          <t>require sponsorship</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -3333,31 +3333,31 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Public Trust</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>reside in the u.s.</t>
+          <t>technical challenge</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>For my selenium based automatic form entry application I was making, I needed it to be flexible enough for different types of DOM structures. I initially started by scraping the relevant types of Web Elements (labels, inputs, buttons, textareas, etc.). This list structure wasn't capturing the hierarchy of the DOM, so I build a node array where the shallow-depth DOM elements are treated as the parent node in the array, and the deeper-depth DOM elements are treated as the parent node's childrent. In the process of figuring this out, I would usually print out the relevant data in the terminal to analyze the order of Web Elements and their Depth, and also sketch possible data structures that could co-relate with with the DOM hierarchy. Link to project: https://github.com/RaqibZaman/AutomateJobApplication</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>work authorization</t>
+          <t>security clearance</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>citizen</t>
+          <t>Public Trust</t>
         </is>
       </c>
     </row>
@@ -3408,17 +3408,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>available to start</t>
+          <t>reside in the u.s.</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -3442,58 +3442,58 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>reason for leaving</t>
+          <t>related experience</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>laid off, end of contract</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>current clearance</t>
+          <t>available to start</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>DHS Public Trust</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>method of contact</t>
+          <t>level of education</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>4 Year University</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>did you graduate?</t>
+          <t>work authorization</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -3503,31 +3503,31 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>citizen</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>18 years or older</t>
+          <t>reason for leaving</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>laid off, end of contract</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>disability status</t>
+          <t>did you graduate?</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -3537,31 +3537,31 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Disability Status</t>
+          <t>current clearance</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>No, I do not have a disability and have not had one in the past</t>
+          <t>DHS Public Trust</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>any accommodation</t>
+          <t>disability status</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -3571,24 +3571,24 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>ethnic background</t>
+          <t>18 years or older</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>asian</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>driver's license</t>
+          <t>method of contact</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -3622,14 +3622,14 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Email</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ts/sci with poly</t>
+          <t>Disability Status</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -3639,48 +3639,48 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>No, I do not have a disability and have not had one in the past</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>able to relocate</t>
+          <t>ethnic background</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Doesn't apply</t>
+          <t>asian</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>select your race</t>
+          <t>any accommodation</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Asian</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>current location</t>
+          <t>years of Back-end</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -3690,27 +3690,31 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Lorton, VA</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Clearance Level</t>
+          <t>select your race</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr"/>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>may we contact?</t>
+          <t>ts/sci with poly</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -3720,48 +3724,48 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>current company</t>
+          <t>reliably commute</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>CVP (Customer Value Partners)</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>recent employer</t>
+          <t>driver's license</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>CVP (Customer Value Partners)</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>date available</t>
+          <t>current location</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -3771,82 +3775,78 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>Lorton, VA</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>elevator pitch</t>
+          <t>able to relocate</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>I’m Raqib Zaman, a detail-oriented full stack software developer with over four years of experience building enterprise web applications, primarily using ASP.NET MVC, C#, JavaScript, and SQL. I specialize in creating accessible, high-quality solutions for federal clients, ensuring compliance with standards like Section 508 while delivering features that improve efficiency and user experience. Beyond development, I have hands-on experience with DevOps tools like Docker and AWS, and have developed automation tools using Python and Selenium to streamline repetitive tasks and improve workflow efficiency. I’m passionate about writing clean, maintainable code that solves real-world problems and drives positive impact.</t>
+          <t>Doesn't apply</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>veteran status</t>
+          <t>why you applied</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>not a protected veteran</t>
+          <t>I'm interested in working with your team because it aligns with my experience building scalable, accessible web applications using ASP.NET MVC, C#, JavaScript, and SQL—especially in federal environments like DHS EPHP DSS and FPS PTS. I enjoy solving real-world problems through full stack development, such as implementing dynamic form logic, exportable reports, and Section 508 compliance. I’m excited by opportunities to contribute to meaningful software that improves user workflows, meets client standards, and supports long-term maintainability.</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>veteran status</t>
+          <t>Clearance Level</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>not a veteran</t>
-        </is>
-      </c>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>current company</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>I am not a veteran</t>
+          <t>CVP (Customer Value Partners)</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>highest degree</t>
+          <t>recent employer</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -3856,14 +3856,14 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Bachelors Degree in Computer Science</t>
+          <t>CVP (Customer Value Partners)</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>united states</t>
+          <t>may we contact?</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -3880,7 +3880,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>how you found</t>
+          <t>date available</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -3890,48 +3890,48 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>indeed.com</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>veteran status</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Apply anyway</t>
+          <t>not a protected veteran</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>cover letter</t>
+          <t>elevator pitch</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>enter text</t>
+          <t>I’m Raqib Zaman, a detail-oriented full stack software developer with over four years of experience building enterprise web applications, primarily using ASP.NET MVC, C#, JavaScript, and SQL. I specialize in creating accessible, high-quality solutions for federal clients, ensuring compliance with standards like Section 508 while delivering features that improve efficiency and user experience. Beyond development, I have hands-on experience with DevOps tools like Docker and AWS, and have developed automation tools using Python and Selenium to streamline repetitive tasks and improve workflow efficiency. I’m passionate about writing clean, maintainable code that solves real-world problems and drives positive impact.</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>I understand</t>
+          <t>Veteran Status</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -3941,48 +3941,48 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>I understand</t>
+          <t>I am not a veteran</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>u.s. citizen</t>
+          <t>highest degree</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Bachelors Degree in Computer Science</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>I understand</t>
+          <t>veteran status</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>checkbox</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>not a veteran</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>shareholder</t>
+          <t>united states</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -3992,63 +3992,65 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>u.s citizen</t>
+          <t>how you found</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>indeed.com</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Desired Pay</t>
+          <t>Apply anyway</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C211" t="n">
-        <v>120000</v>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Apply anyway</t>
+        </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>middle name</t>
+          <t>I understand</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>uz</t>
+          <t>I understand</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>sponsorship</t>
+          <t>cover letter</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -4058,31 +4060,31 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>enter text</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>disability</t>
+          <t>I understand</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>checkbox</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>US Citizen</t>
+          <t>u.s. citizen</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -4099,15 +4101,149 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
+          <t>u.s citizen</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>shareholder</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Desired Pay</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>middle name</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>uz</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Postal Code</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>22079</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>sponsorship</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>US Citizen</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>disability</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
           <t>enter text</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr">
+      <c r="B224" t="inlineStr">
         <is>
           <t>[cover letter]</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr">
+      <c r="C224" t="inlineStr">
         <is>
           <t>Dear Hiring Manager,
 I am writing to express my interest in the Software Developer position at [Company Name], as advertised. With over four years of hands-on experience developing full stack enterprise web applications for federal clients, I bring a strong foundation in ASP.NET MVC, C#, JavaScript, SQL, and accessibility standards. My technical proficiency and dedication to delivering high-quality, compliant software solutions align well with your team’s mission.
@@ -4120,159 +4256,27 @@
         </is>
       </c>
     </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>job title</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>Full Stack Developer</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>Bachelors Degree</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>ethnicity</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>select-one</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>asian</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>ethnicity</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>not</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>you have</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>pronouns</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr"/>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>18 years</t>
-        </is>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Continue</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Continue</t>
+          <t>Bachelors Degree</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>new jobs</t>
+          <t>ethnicity</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -4282,65 +4286,65 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>not</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>I agree</t>
+          <t>ethnicity</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>I understand</t>
+          <t>asian</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>country</t>
+          <t>great fit</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>I’m a great fit for this position because I have a solid track record of delivering end-to-end technical solutions that solve complex problems across the full stack. My experience with ASP.NET MVC, C#, JavaScript, and SQL has allowed me to build scalable, accessible, and maintainable systems for enterprise and federal clients. I approach development with a focus on clean architecture, automation, and performance, using tools like LINQ, Entity Framework, Docker, and AWS to streamline workflows and meet evolving requirements. This position aligns with my passion for solving real-world challenges through code, contributing to impactful systems, and continuously improving both the product and my technical capabilities.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>consent</t>
+          <t>job title</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>i consent</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>citizen</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -4350,93 +4354,95 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>citizen</t>
+          <t>Bachelor</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>salary</t>
+          <t>frequency</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C231" t="n">
-        <v>120000</v>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>yearly</t>
+        </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>suffix</t>
+          <t>new jobs</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C232" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>pronouns</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C233" t="inlineStr">
-        <is>
-          <t>[Male]</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>felony</t>
+          <t>Continue</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>button</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Continue</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>select-one</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>[man]</t>
+          <t>usd</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>limit</t>
+          <t>18 years</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -4446,14 +4452,14 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>agree</t>
+          <t>you have</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -4470,7 +4476,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>country</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -4480,143 +4486,392 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Anytime (8am - 9pm)</t>
+          <t>United States</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Race</t>
+          <t>consent</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Asian</t>
+          <t>i consent</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>citizen</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>[current date]</t>
+          <t>citizen</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>I agree</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Raqib Zaman</t>
+          <t>I understand</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Rate</t>
+          <t>salary</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="C242" t="inlineStr">
-        <is>
-          <t>[average]</t>
-        </is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>okay</t>
+          <t>start?</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>[current date]</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>felony</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Anytime</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>select-one</t>
+          <t>radio</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Weekday</t>
+          <t>[Male]</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>[man]</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>suffix</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>120000</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>virginia</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Raqib Zaman</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>[current date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>okay</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Anytime</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Anytime (8am - 9pm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>[average]</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
           <t>zip</t>
         </is>
       </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C246" t="inlineStr">
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
         <is>
           <t>22079</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>fit</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>I’m a great fit for this position because I have a solid track record of delivering end-to-end technical solutions that solve complex problems across the full stack. My experience with ASP.NET MVC, C#, JavaScript, and SQL has allowed me to build scalable, accessible, and maintainable systems for enterprise and federal clients. I approach development with a focus on clean architecture, automation, and performance, using tools like LINQ, Entity Framework, Docker, and AWS to streamline workflows and meet evolving requirements. This position aligns with my passion for solving real-world challenges through code, contributing to impactful systems, and continuously improving both the product and my technical capabilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>select-one</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Weekday</t>
         </is>
       </c>
     </row>

</xml_diff>